<commit_message>
Spreadsheet met lijst afgetreden bewindspersonen bijgewerkt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GWDzH9CBKYVCbFWmsbqcR
</commit_message>
<xml_diff>
--- a/stamlijsten.xlsx
+++ b/stamlijsten.xlsx
@@ -17,7 +17,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NL politiek &amp; geschiedenis" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wetenschap" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NL films" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzoektips" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Afgetreden bewindspersonen" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzoektips" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -202,6 +203,23 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T0" displayName="T0" ref="A1:H69" headerRowCount="1">
   <autoFilter ref="A1:H69"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Prio"/>
+    <tableColumn id="2" name="Vraag"/>
+    <tableColumn id="3" name="Voorleesvraag"/>
+    <tableColumn id="4" name="Antwoord"/>
+    <tableColumn id="5" name="Extra"/>
+    <tableColumn id="6" name="Afbeelding"/>
+    <tableColumn id="7" name="Wiki"/>
+    <tableColumn id="8" name="Al gevraagd"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T9" displayName="T9" ref="A1:H61" headerRowCount="1">
+  <autoFilter ref="A1:H61"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Prio"/>
     <tableColumn id="2" name="Vraag"/>
@@ -1708,6 +1726,1823 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Prio</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Vraag</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Voorleesvraag</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Antwoord</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Afbeelding</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Wiki</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Al gevraagd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris Toeslagen (NSC), afgetreden nov. 2024 om polariserende uitlatingen van collega's</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>In november 2024 stapte deze NSC-staatssecretaris van Toeslagen en Douane op, omdat ze de polariserende omgangsvormen en uitlatingen van collega's in het kabinet-Schoof niet langer accepteerde. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Nora Achahbar</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Kabinet-Schoof</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr"/>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>Nora Achahbar</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris Fiscaliteit (NSC), afgetreden nov. 2024 om zakelijke belangen</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Deze NSC-staatssecretaris van Fiscaliteit trad in november 2024 af na commotie over het niet openbaar maken van zijn zakelijke belangen. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Folkert Idsinga</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Opgevolgd door Tjebbe van Oostenbrugge</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr"/>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Folkert Idsinga</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Buitenlandse Zaken (NSC), opgestapt aug. 2025 over maatregelen tegen Israël</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Deze minister van Buitenlandse Zaken van NSC stapte in augustus 2025 op omdat hij geen steun kreeg voor extra maatregelen tegen Israël; daarna verliet heel NSC het kabinet-Schoof. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Caspar Veldkamp</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="9" t="inlineStr"/>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Caspar Veldkamp</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Partij die in juni 2025 uit het kabinet-Schoof stapte (asiel)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>In juni 2025 trok deze partij al haar bewindspersonen terug uit het kabinet-Schoof, omdat haar asielmaatregelen niet snel genoeg werden overgenomen. Welke partij was dit?</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>PVV</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Leider Geert Wilders</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr"/>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Partij voor de Vrijheid</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Minister van VWS (D66), vertrok jan. 2024 voor internationale functie</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Deze D66-minister van Volksgezondheid, die het land door de coronacrisis loodste, vertrok in januari 2024 voor een internationale functie. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Ernst Kuipers</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Ernst Kuipers</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Financiën (D66), vertrok jan. 2024 als VN-coördinator Gaza</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Deze minister van Financiën en vicepremier vertrok in januari 2024 om VN-coördinator voor humanitaire hulp in Gaza te worden. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Sigrid Kaag</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Trad in 2021 ook al af als minister van Buitenlandse Zaken</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Sigrid Kaag</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris Cultuur en Media (D66), vertrok dec. 2023</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Deze D66-staatssecretaris voor Cultuur en Media vertrok eind 2023 om terug te keren naar het bedrijfsleven. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Gunay Uslu</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr"/>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Gunay Uslu</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Buitenlandse Zaken (CDA), vertrok aug. 2023 naar Europese Commissie</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-minister van Buitenlandse Zaken en vicepremier vertrok in 2023 naar Brussel om Eurocommissaris voor klimaat te worden, als opvolger van Frans Timmermans. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Wopke Hoekstra</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr"/>
+      <c r="F9" s="9" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Wopke Hoekstra</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Minister Primair en Voortgezet Onderwijs (VVD), afgetreden juni 2023 om intimiderend gedrag</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-minister voor Onderwijs trad in juni 2023 af na herhaalde berichten over intimiderend gedrag en woede-uitbarstingen tegenover ambtenaren. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Dennis Wiersma</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Dennis Wiersma</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Landbouw (ChristenUnie), afgetreden sept. 2022 om stikstof</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Deze ChristenUnie-minister van Landbouw trad na nog geen negen maanden af, omdat hij zichzelf niet de juiste persoon vond om de stikstofcrisis op te lossen. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Henk Staghouwer</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Opgevolgd door Piet Adema</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Henk Staghouwer</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris EZK (CDA), ontslagen sept. 2021 na kritiek op coronapas</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-staatssecretaris van Economische Zaken uitte in een interview openlijk kritiek op de coronapas en werd daarop in september 2021 ontslagen. Ze werd later vicepremier namens BBB. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Mona Keijzer</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr"/>
+      <c r="F12" s="9" t="inlineStr"/>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>Mona Keijzer</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Defensie (CDA), afgetreden sept. 2021 om evacuatie Afghanistan</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-minister van Defensie trad in september 2021 af na een motie van afkeuring over de chaotische evacuatie uit Afghanistan, een dag na haar collega van Buitenlandse Zaken. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Ank Bijleveld</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Samen met Sigrid Kaag</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr"/>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Ank Bijleveld</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Buitenlandse Zaken (D66), afgetreden sept. 2021 om evacuatie Afghanistan</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Na een motie van afkeuring over de evacuatie uit Kabul trad deze D66-minister van Buitenlandse Zaken in september 2021 af; haar collega van Defensie volgde een dag later. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Sigrid Kaag</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Samen met Ank Bijleveld</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr"/>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Sigrid Kaag</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Minister voor Medische Zorg (VVD), afgetreden sept. 2021 om gezondheid</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-minister voor Medische Zorg trad in september 2021 af vanwege gezondheidsproblemen. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Tamara van Ark</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="9" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Tamara van Ark</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Minister van I&amp;W (VVD), vertrok aug. 2021 naar energiebranche</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-minister van Infrastructuur en Waterstaat vertrok in 2021 om voorzitter te worden van de branchevereniging van energiebedrijven. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Cora van Nieuwenhuizen</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr"/>
+      <c r="F16" s="9" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Cora van Nieuwenhuizen</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris I&amp;W (D66), vertrok juli 2021 naar Europees instituut</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Deze D66-staatssecretaris van Infrastructuur en Waterstaat vertrok in 2021 voor een functie bij een Europees instituut en keerde in 2026 terug als minister. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Stientje van Veldhoven</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr"/>
+      <c r="F17" s="9" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Stientje van Veldhoven</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Minister van EZK (VVD), afgetreden jan. 2021 om toeslagenaffaire</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-minister van Economische Zaken trad in januari 2021 direct af, omdat hij eerder als staatssecretaris van Financiën verantwoordelijk was voor de Belastingdienst tijdens de toeslagenaffaire. Hij wachtte de val van het kabinet niet af. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Eric Wiebes</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr"/>
+      <c r="F18" s="9" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Eric Wiebes</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Minister voor Medische Zorg (VVD), afgetreden maart 2020 door oververmoeidheid</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-minister voor Medische Zorg viel in maart 2020 flauw tijdens een Kamerdebat over het coronavirus en trad daarna af wegens oververmoeidheid. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Bruno Bruins</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr"/>
+      <c r="F19" s="9" t="inlineStr"/>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Bruno Bruins</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris van Financiën (D66), afgetreden dec. 2019 om toeslagenaffaire</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Deze D66-staatssecretaris van Financiën trad in december 2019 af over de afhandeling van de kinderopvangtoeslagenaffaire. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Menno Snel</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr"/>
+      <c r="F20" s="9" t="inlineStr"/>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Menno Snel</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris J&amp;V (VVD), afgetreden mei 2019 om onjuist informeren over criminele asielzoekers</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-staatssecretaris van Justitie trad in mei 2019 af omdat hij de Kamer onvolledig had geïnformeerd over misdrijven door asielzoekers. Hij werd later minister van Infrastructuur. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Mark Harbers</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr"/>
+      <c r="F21" s="9" t="inlineStr"/>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Mark Harbers</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Buitenlandse Zaken (VVD), afgetreden feb. 2018 om verzonnen Poetin-verhaal</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-minister van Buitenlandse Zaken trad in februari 2018 af, nadat bleek dat hij had gelogen over zijn aanwezigheid bij een uitspraak van Poetin over 'Groot-Rusland'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Halbe Zijlstra</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr"/>
+      <c r="F22" s="9" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Halbe Zijlstra</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Defensie (VVD), afgetreden okt. 2017 om mortierongeluk Mali</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-minister van Defensie trad in oktober 2017 af na een vernietigend OVV-rapport over het mortierongeluk in Mali, waarbij twee militairen omkwamen. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Jeanine Hennis</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Ook Hennis-Plasschaert; later VN-gezant</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Jeanine Hennis-Plasschaert</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris van Landbouw (PvdA), vertrok sept. 2017 naar de NPO</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-staatssecretaris van Landbouw vertrok in 2017 om bestuurder te worden bij de publieke omroep NPO. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Martijn van Dam</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr"/>
+      <c r="F24" s="9" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Martijn van Dam</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Minister V&amp;J (VVD), afgetreden jan. 2017 om Teevendeal</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-minister van Veiligheid en Justitie trad in januari 2017 af vanwege zijn rol bij het beantwoorden van Kamervragen over de Teevendeal, uit zijn tijd als Kamerlid. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Ard van der Steur</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr"/>
+      <c r="F25" s="9" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Ard van der Steur</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris I&amp;M (PvdA), afgetreden okt. 2015 na Fyra-enquête</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-staatssecretaris van Infrastructuur trad in oktober 2015 af na de uitkomst van de parlementaire enquête naar de mislukte hogesnelheidstrein Fyra. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Wilma Mansveld</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr"/>
+      <c r="F26" s="9" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Wilma Mansveld</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Minister V&amp;J (VVD), afgetreden maart 2015 om bonnetjesaffaire</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-minister van Veiligheid en Justitie trad in maart 2015 samen met zijn staatssecretaris af over de bonnetjesaffaire: de schikking met drugscrimineel Cees H. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Ivo Opstelten</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Samen met Fred Teeven</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Ivo Opstelten</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris V&amp;J (VVD), afgetreden maart 2015 om bonnetjesaffaire</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-staatssecretaris en oud-officier van justitie had in 2000 de schikking met drugscrimineel Cees H. gesloten; in 2015 trad hij af samen met zijn minister. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Fred Teeven</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Samen met Ivo Opstelten</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Fred Teeven</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Buitenlandse Zaken (PvdA), vertrok 2014 naar Europese Commissie</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-minister van Buitenlandse Zaken, bekend van zijn toespraak bij de VN over de MH17-ramp, vertrok in 2014 als eerste vicevoorzitter naar de Europese Commissie. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Frans Timmermans</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr"/>
+      <c r="F29" s="9" t="inlineStr"/>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Frans Timmermans</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris van Financiën (VVD), afgetreden jan. 2014 om toeslagenproblemen</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-staatssecretaris van Financiën trad in januari 2014 af na problemen bij de uitbetaling van toeslagen door de Belastingdienst. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Frans Weekers</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr"/>
+      <c r="F30" s="9" t="inlineStr"/>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Frans Weekers</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris VWS (PvdA), na 3 weken afgetreden dec. 2012 om declaraties</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-staatssecretaris van Volksgezondheid trad al na drie weken af, in december 2012, vanwege onjuiste reiskostendeclaraties uit zijn tijd als gedeputeerde in Gelderland. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Co Verdaas</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr"/>
+      <c r="F31" s="9" t="inlineStr"/>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Co Verdaas</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Minister BZK (CDA), vertrok 2011 naar de Raad van State</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-minister van Binnenlandse Zaken vertrok eind 2011 om vicepresident van de Raad van State te worden. Hij was in 2006 ook al afgetreden als minister van Justitie. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Piet Hein Donner</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr"/>
+      <c r="F32" s="9" t="inlineStr"/>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Piet Hein Donner</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris van Defensie (CDA), afgetreden mei 2010 om relatie met ondergeschikte</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-staatssecretaris van Defensie, eerder campagneleider van het CDA, trad in mei 2010 af na een relatie met een ondergeschikte. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Jack de Vries</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr"/>
+      <c r="F33" s="9" t="inlineStr"/>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Jack de Vries</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Partij die in 2010 om de missie in Uruzgan uit het kabinet stapte</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>In februari 2010 stapten alle bewindspersonen van deze partij uit het vierde kabinet-Balkenende vanwege een conflict over verlenging van de militaire missie in Uruzgan. Welke partij?</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>PvdA</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Leider Wouter Bos</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr"/>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Partij van de Arbeid</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris SZW (PvdA), vertrok 2008 als burgemeester van Rotterdam</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-staatssecretaris van Sociale Zaken vertrok eind 2008 om burgemeester van Rotterdam te worden. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Ahmed Aboutaleb</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr"/>
+      <c r="F35" s="9" t="inlineStr"/>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Ahmed Aboutaleb</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Minister voor Wonen, Wijken en Integratie (PvdA), afgetreden nov. 2008</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-minister voor Wonen, Wijken en Integratie, bekend van de 'krachtwijken', trad in november 2008 af na kritiek op haar functioneren uit haar eigen partij. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Ella Vogelaar</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr"/>
+      <c r="F36" s="9" t="inlineStr"/>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Ella Vogelaar</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris van Defensie (CDA), vertrok 2007 als burgemeester van Ede</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-staatssecretaris van Defensie vertrok eind 2007 om burgemeester van Ede te worden. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Cees van der Knaap</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr"/>
+      <c r="F37" s="9" t="inlineStr"/>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Cees van der Knaap</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Minister van VROM (VVD), afgetreden sept. 2006 om Schipholbrand</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-minister van Volkshuisvesting trad in september 2006 af na het OVV-rapport over de brand in het detentiecentrum Schiphol-Oost, waarbij elf mensen omkwamen. Haar collega van Justitie trad gelijk met haar af. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Sybilla Dekker</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Samen met Piet Hein Donner</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr"/>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>Sybilla Dekker</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Justitie (CDA), afgetreden sept. 2006 om Schipholbrand</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-minister van Justitie trad in september 2006 af na het OVV-rapport over de dodelijke brand in het cellencomplex bij Schiphol-Oost. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Piet Hein Donner</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Samen met Sybilla Dekker</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr"/>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Piet Hein Donner</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris OCW (VVD), vertrok 2006 om VVD-fractievoorzitter te worden</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-staatssecretaris van Onderwijs vertrok in juni 2006 om fractievoorzitter van de VVD te worden. Later werd hij de langstzittende premier ooit. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Mark Rutte</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr"/>
+      <c r="F40" s="9" t="inlineStr"/>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Mark Rutte</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Minister Bestuurlijke Vernieuwing (D66), afgetreden 2005 om gekozen burgemeester</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Deze D66-minister trad in maart 2005 af toen de Eerste Kamer zijn grondwetsvoorstel voor de gekozen burgemeester verwierp. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Thom de Graaf</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr"/>
+      <c r="F41" s="9" t="inlineStr"/>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Thom de Graaf</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris OCW (VVD), afgetreden 2004 door slechte verhouding met minister</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-staatssecretaris van Onderwijs trad in 2004 af door een slechte verhouding met haar minister Maria van der Hoeven. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Annette Nijs</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr"/>
+      <c r="F42" s="9" t="inlineStr"/>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>Annette Nijs</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Buitenlandse Zaken (CDA), vertrok 2003 naar de NAVO</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-minister van Buitenlandse Zaken vertrok eind 2003 om secretaris-generaal van de NAVO te worden. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Jaap de Hoop Scheffer</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr"/>
+      <c r="F43" s="9" t="inlineStr"/>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Jaap de Hoop Scheffer</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Defensie (VVD), afgetreden dec. 2002 na bouwfraude-enquête</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-minister van Defensie trad in december 2002 af na de uitkomst van de parlementaire enquête naar de bouwfraude, over zijn eerdere rol als minister van Justitie. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Benk Korthals</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr"/>
+      <c r="F44" s="9" t="inlineStr"/>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>Benk Korthals</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Minister van VWS (LPF), opgestapt okt. 2002 door ruzie met collega</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>In oktober 2002 stapten twee ruziënde LPF-ministers op, waarna het eerste kabinet-Balkenende viel. Deze econoom was minister van Volksgezondheid. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Eduard Bomhoff</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Ruzie met Herman Heinsbroek</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr"/>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>Eduard Bomhoff</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Minister van EZ (LPF), opgestapt okt. 2002 door ruzie met collega</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>In oktober 2002 stapten twee ruziënde LPF-ministers op. Deze zakenman, oprichter van een platenmaatschappij, was minister van Economische Zaken. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Herman Heinsbroek</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>Ruzie met Eduard Bomhoff</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr"/>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>Herman Heinsbroek</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris Emancipatie (LPF), afgetreden juli 2002 op de eerste dag</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Deze LPF-staatssecretaris van Emancipatie trad in juli 2002 al op haar eerste werkdag af, na onthullingen over haar verleden in een Surinaamse militie. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Philomena Bijlhout</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr"/>
+      <c r="F47" s="9" t="inlineStr"/>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>Philomena Bijlhout</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris van Justitie (PvdA), vertrok 2001 als burgemeester van Amsterdam</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-staatssecretaris van Justitie, bekend van de nieuwe Vreemdelingenwet, vertrok begin 2001 om burgemeester van Amsterdam te worden. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Job Cohen</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr"/>
+      <c r="F48" s="9" t="inlineStr"/>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>Job Cohen</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Minister BZK (PvdA), afgetreden maart 2000 om declaraties als burgemeester</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-minister van Binnenlandse Zaken trad in maart 2000 af nadat hij in opspraak kwam over zijn declaraties als burgemeester van Rotterdam. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Bram Peper</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr"/>
+      <c r="F49" s="9" t="inlineStr"/>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>Bram Peper</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Landbouw (D66), afgetreden juni 1999</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Deze D66-minister van Landbouw trad in juni 1999 af, omdat hij ontevreden was over zijn beleidsmogelijkheden. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Hayo Apotheker</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr"/>
+      <c r="F50" s="9" t="inlineStr"/>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>Hayo Apotheker</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris SZW (VVD), afgetreden juni 1996 om CTSV-affaire</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Deze VVD-staatssecretaris van Sociale Zaken trad in juni 1996 af vanwege de CTSV-affaire, over het toezicht op de sociale zekerheid. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Robin Linschoten</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr"/>
+      <c r="F51" s="9" t="inlineStr"/>
+      <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>Robin Linschoten</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Minister van WVC (PvdA), vertrok 1994 naar Europees Parlement</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-minister van Welzijn, Volksgezondheid en Cultuur vertrok in 1994 naar het Europees Parlement, samen met haar CDA-collega van Verkeer en Waterstaat. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Hedy d'Ancona</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr"/>
+      <c r="F52" s="9" t="inlineStr"/>
+      <c r="G52" s="8" t="inlineStr">
+        <is>
+          <t>Hedy d'Ancona</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Minister van V&amp;W (CDA), vertrok 1994 naar Europees Parlement</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-minister van Verkeer en Waterstaat vertrok in 1994 naar het Europees Parlement. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Hanja Maij-Weggen</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr"/>
+      <c r="F53" s="9" t="inlineStr"/>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>Hanja Maij-Weggen</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Justitie (CDA), afgetreden mei 1994 om IRT-affaire</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-minister van Justitie trad in mei 1994 af over de IRT-affaire, rond omstreden opsporingsmethoden; zijn collega van Binnenlandse Zaken trad met hem af. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Ernst Hirsch Ballin</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Samen met Ed van Thijn</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="inlineStr"/>
+      <c r="G54" s="8" t="inlineStr">
+        <is>
+          <t>Ernst Hirsch Ballin</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Minister BZK (PvdA), afgetreden mei 1994 om IRT-affaire</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-minister van Binnenlandse Zaken, oud-burgemeester van Amsterdam, trad in mei 1994 af over de IRT-affaire. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Ed van Thijn</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Samen met Ernst Hirsch Ballin</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr"/>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>Ed van Thijn</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris WVC (PvdA), vertrok 1994 als lijsttrekker in Rotterdam</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-staatssecretaris van Welzijn, Volksgezondheid en Cultuur vertrok in 1994 om lijsttrekker te worden bij de gemeenteraadsverkiezingen in Rotterdam. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Hans Simons</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr"/>
+      <c r="F56" s="9" t="inlineStr"/>
+      <c r="G56" s="8" t="inlineStr">
+        <is>
+          <t>Hans Simons</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris O&amp;W (PvdA), afgetreden 1993 om nevenfuncties</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-staatssecretaris van Onderwijs trad in 1993 af nadat hij in opspraak kwam over zijn nevenfuncties. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Roel in 't Veld</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr"/>
+      <c r="F57" s="9" t="inlineStr"/>
+      <c r="G57" s="8" t="inlineStr">
+        <is>
+          <t>Roel in 't Veld</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris SZW (PvdA), afgetreden 1993 door spanningen met de fractie</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Deze PvdA-staatssecretaris van Sociale Zaken trad in 1993 af door spanningen met de PvdA-fractie. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Elske ter Veld</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr"/>
+      <c r="F58" s="9" t="inlineStr"/>
+      <c r="G58" s="8" t="inlineStr">
+        <is>
+          <t>Elske ter Veld</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Staatssecretaris van Defensie (CDA), vertrok 1993 als gouverneur van Limburg</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-staatssecretaris van Defensie vertrok in 1993 om Commissaris van de Koningin in Limburg te worden. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Berend-Jan van Voorst tot Voorst</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr"/>
+      <c r="F59" s="9" t="inlineStr"/>
+      <c r="G59" s="8" t="inlineStr">
+        <is>
+          <t>Berend-Jan van Voorst tot Voorst</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Buitenlandse Zaken (CDA), vertrok 1993 naar Europese Commissie</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-minister van Buitenlandse Zaken vertrok begin 1993 om lid te worden van de Europese Commissie. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Hans van den Broek</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr"/>
+      <c r="F60" s="9" t="inlineStr"/>
+      <c r="G60" s="8" t="inlineStr">
+        <is>
+          <t>Hans van den Broek</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Minister van Landbouw (CDA), afgetreden 1990 om visfraude</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Deze CDA-minister van Landbouw trad in september 1990 af, nadat hij het vertrouwen van de PvdA-fractie verloor over zijn beleid tegen visfraude. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Gerrit Braks</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr"/>
+      <c r="F61" s="9" t="inlineStr"/>
+      <c r="G61" s="8" t="inlineStr">
+        <is>
+          <t>Gerrit Braks</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Nieuwe lijst: Songfestival-winnaars 2010-2026 (artiest, nummer, land)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GWDzH9CBKYVCbFWmsbqcR
</commit_message>
<xml_diff>
--- a/stamlijsten.xlsx
+++ b/stamlijsten.xlsx
@@ -18,7 +18,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Wetenschap" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NL films" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Afgetreden bewindspersonen" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzoektips" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Songfestival" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzoektips" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -220,6 +221,23 @@
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T9" displayName="T9" ref="A1:H61" headerRowCount="1">
   <autoFilter ref="A1:H61"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Prio"/>
+    <tableColumn id="2" name="Vraag"/>
+    <tableColumn id="3" name="Voorleesvraag"/>
+    <tableColumn id="4" name="Antwoord"/>
+    <tableColumn id="5" name="Extra"/>
+    <tableColumn id="6" name="Afbeelding"/>
+    <tableColumn id="7" name="Wiki"/>
+    <tableColumn id="8" name="Al gevraagd"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="T10" displayName="T10" ref="A1:H50" headerRowCount="1">
+  <autoFilter ref="A1:H50"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Prio"/>
     <tableColumn id="2" name="Vraag"/>
@@ -3543,6 +3561,1651 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Prio</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Vraag</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Voorleesvraag</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Antwoord</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Afbeelding</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Wiki</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Al gevraagd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2010: winnende artiest (Duitsland)</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2010 werd gehouden in Oslo en gewonnen door Duitsland. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Lena</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>2010: Lena – Satellite (Duitsland); gaststad Oslo</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr"/>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>Lena Meyer-Landrut</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2010: winnend nummer van Lena</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>In 2010, in Oslo, won Lena het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Satellite</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>2010: Lena – Satellite (Duitsland); gaststad Oslo</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr"/>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>?Satellite Lena Eurovisie</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2010: winnend land ('Satellite')</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2010 in Oslo, met het nummer 'Satellite'?</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Duitsland</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>2010: Lena – Satellite (Duitsland); gaststad Oslo</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr"/>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2010</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2011: winnende artiest (Azerbeidzjan)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2011 werd gehouden in Düsseldorf en gewonnen door Azerbeidzjan. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Ell &amp; Nikki</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>2011: Ell &amp; Nikki – Running Scared (Azerbeidzjan); gaststad Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr"/>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Ell &amp; Nikki</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2011: winnend nummer van Ell &amp; Nikki</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>In 2011, in Düsseldorf, won Ell &amp; Nikki het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Running Scared</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>2011: Ell &amp; Nikki – Running Scared (Azerbeidzjan); gaststad Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>?Running Scared Ell &amp; Nikki Eurovisie</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2011: winnend land ('Running Scared')</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2011 in Düsseldorf, met het nummer 'Running Scared'?</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Azerbeidzjan</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>2011: Ell &amp; Nikki – Running Scared (Azerbeidzjan); gaststad Düsseldorf</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2011</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2012: winnende artiest (Zweden)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2012 werd gehouden in Bakoe en gewonnen door Zweden. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Loreen</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>2012: Loreen – Euphoria (Zweden); gaststad Bakoe</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr"/>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Loreen</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2012: winnend nummer van Loreen</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>In 2012, in Bakoe, won Loreen het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Euphoria</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>2012: Loreen – Euphoria (Zweden); gaststad Bakoe</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>?Euphoria Loreen Eurovisie</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2012: winnend land ('Euphoria')</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2012 in Bakoe, met het nummer 'Euphoria'?</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Zweden</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>2012: Loreen – Euphoria (Zweden); gaststad Bakoe</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2012</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2013: winnende artiest (Denemarken)</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2013 werd gehouden in Malmö en gewonnen door Denemarken. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Emmelie de Forest</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>2013: Emmelie de Forest – Only Teardrops (Denemarken); gaststad Malmö</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Emmelie de Forest</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2013: winnend nummer van Emmelie de Forest</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>In 2013, in Malmö, won Emmelie de Forest het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Only Teardrops</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>2013: Emmelie de Forest – Only Teardrops (Denemarken); gaststad Malmö</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr"/>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>?Only Teardrops Emmelie de Forest Eurovisie</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2013: winnend land ('Only Teardrops')</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2013 in Malmö, met het nummer 'Only Teardrops'?</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Denemarken</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>2013: Emmelie de Forest – Only Teardrops (Denemarken); gaststad Malmö</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr"/>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2013</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2014: winnende artiest (Oostenrijk)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2014 werd gehouden in Kopenhagen en gewonnen door Oostenrijk. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Conchita Wurst</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>2014: Conchita Wurst – Rise Like a Phoenix (Oostenrijk); gaststad Kopenhagen</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr"/>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>Conchita Wurst</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2014: winnend nummer van Conchita Wurst</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>In 2014, in Kopenhagen, won Conchita Wurst het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Rise Like a Phoenix</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>2014: Conchita Wurst – Rise Like a Phoenix (Oostenrijk); gaststad Kopenhagen</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>?Rise Like a Phoenix Conchita Wurst Eurovisie</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2014: winnend land ('Rise Like a Phoenix')</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2014 in Kopenhagen, met het nummer 'Rise Like a Phoenix'?</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Oostenrijk</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>2014: Conchita Wurst – Rise Like a Phoenix (Oostenrijk); gaststad Kopenhagen</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2014</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2015: winnende artiest (Zweden)</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2015 werd gehouden in Wenen en gewonnen door Zweden. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Måns Zelmerlöw</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>2015: Måns Zelmerlöw – Heroes (Zweden); gaststad Wenen</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Måns Zelmerlöw</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2015: winnend nummer van Måns Zelmerlöw</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>In 2015, in Wenen, won Måns Zelmerlöw het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Heroes</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>2015: Måns Zelmerlöw – Heroes (Zweden); gaststad Wenen</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>?Heroes Måns Zelmerlöw Eurovisie</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2015: winnend land ('Heroes')</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2015 in Wenen, met het nummer 'Heroes'?</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Zweden</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>2015: Måns Zelmerlöw – Heroes (Zweden); gaststad Wenen</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr"/>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2015</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2016: winnende artiest (Oekraïne)</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2016 werd gehouden in Stockholm en gewonnen door Oekraïne. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Jamala</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>2016: Jamala – 1944 (Oekraïne); gaststad Stockholm</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr"/>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>Jamala</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2016: winnend nummer van Jamala</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>In 2016, in Stockholm, won Jamala het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>1944</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>2016: Jamala – 1944 (Oekraïne); gaststad Stockholm</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr"/>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>?1944 Jamala Eurovisie</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2016: winnend land ('1944')</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2016 in Stockholm, met het nummer '1944'?</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Oekraïne</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>2016: Jamala – 1944 (Oekraïne); gaststad Stockholm</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2016</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2017: winnende artiest (Portugal)</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2017 werd gehouden in Kyiv en gewonnen door Portugal. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Salvador Sobral</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>2017: Salvador Sobral – Amar pelos dois (Portugal); gaststad Kyiv</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Salvador Sobral</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2017: winnend nummer van Salvador Sobral</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>In 2017, in Kyiv, won Salvador Sobral het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Amar pelos dois</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>2017: Salvador Sobral – Amar pelos dois (Portugal); gaststad Kyiv</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>?Amar pelos dois Salvador Sobral Eurovisie</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2017: winnend land ('Amar pelos dois')</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2017 in Kyiv, met het nummer 'Amar pelos dois'?</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>2017: Salvador Sobral – Amar pelos dois (Portugal); gaststad Kyiv</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2017</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2018: winnende artiest (Israël)</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2018 werd gehouden in Lissabon en gewonnen door Israël. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Netta</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>2018: Netta – Toy (Israël); gaststad Lissabon</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Netta Barzilai</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2018: winnend nummer van Netta</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>In 2018, in Lissabon, won Netta het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Toy</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>2018: Netta – Toy (Israël); gaststad Lissabon</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>?Toy Netta Eurovisie</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2018: winnend land ('Toy')</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2018 in Lissabon, met het nummer 'Toy'?</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Israël</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>2018: Netta – Toy (Israël); gaststad Lissabon</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2018</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2019: winnende artiest (Nederland)</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2019 werd gehouden in Tel Aviv en gewonnen door Nederland. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Duncan Laurence</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>2019: Duncan Laurence – Arcade (Nederland); gaststad Tel Aviv</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr"/>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Duncan Laurence</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2019: winnend nummer van Duncan Laurence</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>In 2019, in Tel Aviv, won Duncan Laurence het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Arcade</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>2019: Duncan Laurence – Arcade (Nederland); gaststad Tel Aviv</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr"/>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>?Arcade Duncan Laurence Eurovisie</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2019: winnend land ('Arcade')</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2019 in Tel Aviv, met het nummer 'Arcade'?</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>2019: Duncan Laurence – Arcade (Nederland); gaststad Tel Aviv</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr"/>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2019</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2021: winnende artiest (Italië)</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2021 werd gehouden in Rotterdam en gewonnen door Italië. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Måneskin</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>2021: Måneskin – Zitti e buoni (Italië); gaststad Rotterdam</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr"/>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Måneskin</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2021: winnend nummer van Måneskin</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>In 2021, in Rotterdam, won Måneskin het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Zitti e buoni</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>2021: Måneskin – Zitti e buoni (Italië); gaststad Rotterdam</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr"/>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>?Zitti e buoni Måneskin Eurovisie</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2021: winnend land ('Zitti e buoni')</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2021 in Rotterdam, met het nummer 'Zitti e buoni'?</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Italië</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>2021: Måneskin – Zitti e buoni (Italië); gaststad Rotterdam</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr"/>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2021</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2022: winnende artiest (Oekraïne)</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2022 werd gehouden in Turijn en gewonnen door Oekraïne. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Kalush Orchestra</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>2022: Kalush Orchestra – Stefania (Oekraïne); gaststad Turijn</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr"/>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Kalush Orchestra</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2022: winnend nummer van Kalush Orchestra</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>In 2022, in Turijn, won Kalush Orchestra het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Stefania</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>2022: Kalush Orchestra – Stefania (Oekraïne); gaststad Turijn</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr"/>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>?Stefania Kalush Orchestra Eurovisie</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2022: winnend land ('Stefania')</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2022 in Turijn, met het nummer 'Stefania'?</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Oekraïne</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>2022: Kalush Orchestra – Stefania (Oekraïne); gaststad Turijn</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr"/>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2022</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2023: winnende artiest (Zweden)</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2023 werd gehouden in Liverpool en gewonnen door Zweden. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Loreen</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>2023: Loreen – Tattoo (Zweden); gaststad Liverpool</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr"/>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>Loreen</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2023: winnend nummer van Loreen</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>In 2023, in Liverpool, won Loreen het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Tattoo</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>2023: Loreen – Tattoo (Zweden); gaststad Liverpool</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr"/>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>?Tattoo Loreen Eurovisie</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2023: winnend land ('Tattoo')</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2023 in Liverpool, met het nummer 'Tattoo'?</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Zweden</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>2023: Loreen – Tattoo (Zweden); gaststad Liverpool</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr"/>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2023</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2024: winnende artiest (Zwitserland)</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2024 werd gehouden in Malmö en gewonnen door Zwitserland. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Nemo</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>2024: Nemo – The Code (Zwitserland); gaststad Malmö</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr"/>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>Nemo (zanger)</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2024: winnend nummer van Nemo</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>In 2024, in Malmö, won Nemo het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>The Code</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>2024: Nemo – The Code (Zwitserland); gaststad Malmö</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr"/>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>?The Code Nemo Eurovisie</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2024: winnend land ('The Code')</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2024 in Malmö, met het nummer 'The Code'?</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Zwitserland</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>2024: Nemo – The Code (Zwitserland); gaststad Malmö</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr"/>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2024</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2025: winnende artiest (Oostenrijk)</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2025 werd gehouden in Bazel en gewonnen door Oostenrijk. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>JJ</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>2025: JJ – Wasted Love (Oostenrijk); gaststad Bazel</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr"/>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>JJ (zanger)</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2025: winnend nummer van JJ</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>In 2025, in Bazel, won JJ het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Wasted Love</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>2025: JJ – Wasted Love (Oostenrijk); gaststad Bazel</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr"/>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>?Wasted Love JJ Eurovisie</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2025: winnend land ('Wasted Love')</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2025 in Bazel, met het nummer 'Wasted Love'?</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Oostenrijk</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>2025: JJ – Wasted Love (Oostenrijk); gaststad Bazel</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr"/>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2025</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2026: winnende artiest (Bulgarije)</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2026 werd gehouden in Wenen en gewonnen door Bulgarije. Welke artiest of groep won?</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Dara</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>2026: Dara – Bangaranga (Bulgarije); gaststad Wenen</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr"/>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>Dara (zangeres)</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2026: winnend nummer van Dara</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>In 2026, in Wenen, won Dara het Eurovisie Songfestival. Hoe heette het winnende nummer?</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Bangaranga</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>2026: Dara – Bangaranga (Bulgarije); gaststad Wenen</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr"/>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>?Bangaranga Dara Eurovisie</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2026: winnend land ('Bangaranga')</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Welk land won het Eurovisie Songfestival van 2026 in Wenen, met het nummer 'Bangaranga'?</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Bulgarije</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>2026: Dara – Bangaranga (Bulgarije); gaststad Wenen</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr"/>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2026</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Songfestival 2020</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Het Eurovisie Songfestival van 2020 zou in Rotterdam worden gehouden, maar werd afgelast. Waardoor?</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Corona</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Rotterdam hield het festival alsnog in 2021</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr"/>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>Eurovisiesongfestival 2020</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Songfestival: vraag over 2020 verwijderd
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GWDzH9CBKYVCbFWmsbqcR
</commit_message>
<xml_diff>
--- a/stamlijsten.xlsx
+++ b/stamlijsten.xlsx
@@ -236,8 +236,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="T10" displayName="T10" ref="A1:H50" headerRowCount="1">
-  <autoFilter ref="A1:H50"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="T10" displayName="T10" ref="A1:H49" headerRowCount="1">
+  <autoFilter ref="A1:H49"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Prio"/>
     <tableColumn id="2" name="Vraag"/>
@@ -3561,7 +3561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5159,38 +5159,6 @@
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B50" s="7" t="inlineStr">
-        <is>
-          <t>Songfestival 2020</t>
-        </is>
-      </c>
-      <c r="C50" s="7" t="inlineStr">
-        <is>
-          <t>Het Eurovisie Songfestival van 2020 zou in Rotterdam worden gehouden, maar werd afgelast. Waardoor?</t>
-        </is>
-      </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>Corona</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr">
-        <is>
-          <t>Rotterdam hield het festival alsnog in 2021</t>
-        </is>
-      </c>
-      <c r="F50" s="9" t="inlineStr"/>
-      <c r="G50" s="8" t="inlineStr">
-        <is>
-          <t>Eurovisiesongfestival 2020</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Nieuwe lijst: literatuurprijzen 2016-2026 met sfeerbeelden zonder titel/auteur
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GWDzH9CBKYVCbFWmsbqcR
</commit_message>
<xml_diff>
--- a/stamlijsten.xlsx
+++ b/stamlijsten.xlsx
@@ -19,7 +19,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NL films" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Afgetreden bewindspersonen" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Songfestival" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzoektips" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literatuurprijzen" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzoektips" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -238,6 +239,23 @@
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="T10" displayName="T10" ref="A1:H49" headerRowCount="1">
   <autoFilter ref="A1:H49"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Prio"/>
+    <tableColumn id="2" name="Vraag"/>
+    <tableColumn id="3" name="Voorleesvraag"/>
+    <tableColumn id="4" name="Antwoord"/>
+    <tableColumn id="5" name="Extra"/>
+    <tableColumn id="6" name="Afbeelding"/>
+    <tableColumn id="7" name="Wiki"/>
+    <tableColumn id="8" name="Al gevraagd"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T11" displayName="T11" ref="A1:H65" headerRowCount="1">
+  <autoFilter ref="A1:H65"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Prio"/>
     <tableColumn id="2" name="Vraag"/>
@@ -5174,6 +5192,2139 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Prio</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Vraag</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Voorleesvraag</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Antwoord</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Afbeelding</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Wiki</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Al gevraagd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Nobelprijs Literatuur 2016</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>De Nobelprijs voor de Literatuur van 2016 ging naar een Amerikaanse singer-songwriter, als eerste musicus. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Bob Dylan</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>2016: Amerikaanse singer-songwriter; geprezen om nieuwe poëtische expressie binnen de Amerikaanse liedtraditie</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr"/>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>!harmonica blues</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Nobelprijs Literatuur 2017</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>De Nobelprijs voor de Literatuur van 2017 ging naar een Britse romanschrijver die in Japan werd geboren. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Kazuo Ishiguro</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>2017: Brits schrijver, geboren in Japan; o.a. The Remains of the Day en Never Let Me Go</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr"/>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>!English country house</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Nobelprijs Literatuur 2018</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>De Nobelprijs voor de Literatuur van 2018 ging naar een Poolse schrijfster; haar prijs werd een jaar later uitgereikt. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Olga Tokarczuk</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>2018: Poolse schrijfster; de prijs werd pas in 2019 uitgereikt na een schandaal bij de Zweedse Academie</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr"/>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>!Białowieża Forest</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Nobelprijs Literatuur 2019</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>De Nobelprijs voor de Literatuur van 2019 ging naar een Oostenrijkse schrijver en toneelauteur. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Peter Handke</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>2019: Oostenrijkse schrijver en toneelauteur; omstreden om zijn houding in de Joegoslavische oorlogen</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr"/>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>!Austrian Alps village</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Nobelprijs Literatuur 2020</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>De Nobelprijs voor de Literatuur van 2020 ging naar een Amerikaanse dichteres. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Louise Glück</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>2020: Amerikaanse dichteres, o.a. de bundel The Wild Iris</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>!wild iris flower</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Nobelprijs Literatuur 2021</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>De Nobelprijs voor de Literatuur van 2021 ging naar een schrijver die op Zanzibar werd geboren en in Engeland woont. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Abdulrazak Gurnah</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>2021: Tanzaniaans-Britse schrijver, geboren op Zanzibar; schrijft over kolonialisme en vluchtelingen</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>!Stone Town Zanzibar</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Nobelprijs Literatuur 2022</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>De Nobelprijs voor de Literatuur van 2022 ging naar een Franse schrijfster van autobiografisch werk. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Annie Ernaux</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>2022: Franse schrijfster van autobiografisch werk, o.a. De jaren</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr"/>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>!Normandy village street</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Nobelprijs Literatuur 2023</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>De Nobelprijs voor de Literatuur van 2023 ging naar een Noorse toneelschrijver en romancier. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Jon Fosse</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>2023: Noorse toneelschrijver en romancier, o.a. de Septologie</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>!Norwegian fjord</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Nobelprijs Literatuur 2024</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>De Nobelprijs voor de Literatuur van 2024 ging naar een Zuid-Koreaanse schrijfster, als eerste Aziatische vrouw. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Han Kang</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>2024: Zuid-Koreaanse schrijfster, o.a. De vegetariër</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>!Seoul street</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Nobelprijs Literatuur 2025</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>De Nobelprijs voor de Literatuur van 2025 ging naar een Hongaarse schrijver van lange, apocalyptische romans. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>László Krasznahorkai</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>2025: Hongaarse schrijver, o.a. Satanstango, verfilmd door Béla Tarr</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>!Hungarian plain puszta</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Nobelprijs Literatuur 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>De Nobelprijs voor de Literatuur van 2026 ging naar een Canadese dichteres en classica. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Anne Carson</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>2026: Canadese dichteres en classica</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr"/>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>!Greek temple ruins</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>P.C. Hooft-prijs 2016 (verhalend proza)</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>De P.C. Hooft-prijs van 2016, voor verhalend proza, ging naar een Surinaams-Nederlandse schrijfster. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Astrid Roemer</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>2016, verhalend proza: Surinaams-Nederlandse schrijfster, als eerste Surinaamse auteur</t>
+        </is>
+      </c>
+      <c r="F13" s="9" t="inlineStr"/>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>!Paramaribo</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>P.C. Hooft-prijs 2017 (beschouwend proza)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>De P.C. Hooft-prijs van 2017, voor beschouwend proza, ging naar een essayist en NRC-columnist. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Bas Heijne</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>2017, beschouwend proza: essayist en NRC-columnist</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr"/>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>!newspaper reading</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>P.C. Hooft-prijs 2018 (poëzie)</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>De P.C. Hooft-prijs van 2018, voor poëzie, ging naar een dichter en hoogleraar economie. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Nachoem Wijnberg</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>2018, poëzie: dichter en hoogleraar economie</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>!Amsterdam canal autumn</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>P.C. Hooft-prijs 2019 (verhalend proza)</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>De P.C. Hooft-prijs van 2019, voor verhalend proza, ging naar een schrijfster van Het bittere kruid. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Marga Minco</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>2019, verhalend proza: schrijfster van Het bittere kruid</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>!Kamp Westerbork</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>P.C. Hooft-prijs 2020 (beschouwend proza)</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>De P.C. Hooft-prijs van 2020, voor beschouwend proza, ging naar een filosoof. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Maxim Februari</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>2020, beschouwend proza: filosoof, jurist en columnist</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>!law library books</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>P.C. Hooft-prijs 2021 (poëzie)</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>De P.C. Hooft-prijs van 2021, voor poëzie, ging naar een dichter die lang in Zuid-Afrika woonde. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Alfred Schaffer</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>2021, poëzie: dichter die lang in Zuid-Afrika woonde</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>!Cape Town</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>P.C. Hooft-prijs 2022 (verhalend proza)</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>De P.C. Hooft-prijs van 2022, voor verhalend proza, ging naar een romancier van o.a. Blauwe maandagen en Tirza. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Arnon Grunberg</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>2022, verhalend proza: romancier van o.a. Blauwe maandagen en Tirza</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr"/>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>!New York street</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>P.C. Hooft-prijs 2023 (beschouwend proza)</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>De P.C. Hooft-prijs van 2023, voor beschouwend proza, ging naar een schrijver en evolutiebioloog van Darwins dromen. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Tijs Goldschmidt</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>2023, beschouwend proza: schrijver en evolutiebioloog van Darwins dromen</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr"/>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>!cichlid Lake Victoria</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>P.C. Hooft-prijs 2024 (poëzie)</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>De P.C. Hooft-prijs van 2024, voor poëzie, ging naar een eigenzinnige dichteres. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Astrid Lampe</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>2024, poëzie: eigenzinnige dichteres</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr"/>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>!collage art</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>P.C. Hooft-prijs 2025 (verhalend proza)</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>De P.C. Hooft-prijs van 2025, voor verhalend proza, ging naar een meesterverteller uit Maassluis. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Maarten 't Hart</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>2025, verhalend proza: meesterverteller uit Maassluis, o.a. Een vlucht regenwulpen</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>!Maassluis</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>P.C. Hooft-prijs 2026 (beschouwend proza)</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>De P.C. Hooft-prijs van 2026, voor beschouwend proza, ging naar een feministe en activiste; als eerste vrouw winnaar in deze categorie. Wie is dit?</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Anja Meulenbelt</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>2026, beschouwend proza: feministe en activiste; als eerste vrouw winnaar in deze categorie</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>!feminist demonstration 1970s</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2016: titel van Connie Palmen</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Connie Palmen de Libris Literatuur Prijs van 2016? Het boek gaat over het huwelijk van Ted Hughes en Sylvia Plath.</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Jij zegt het</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2016: Connie Palmen – Jij zegt het</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>!Dartmoor landscape</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2016: schrijver van 'Jij zegt het'</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Libris Literatuur Prijs van 2016 met de roman 'Jij zegt het'?</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Connie Palmen</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2016: Connie Palmen – Jij zegt het</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>!Dartmoor landscape</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2017: titel van Alfred Birney</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Alfred Birney de Libris Literatuur Prijs van 2017? Het boek gaat over een Indische vader en de koloniale oorlog.</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>De tolk van Java</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2017: Alfred Birney – De tolk van Java</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>!Java rice field</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2017: schrijver van 'De tolk van Java'</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Libris Literatuur Prijs van 2017 met de roman 'De tolk van Java'?</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Alfred Birney</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2017: Alfred Birney – De tolk van Java</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>!Java rice field</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2018: titel van Murat Isik</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Murat Isik de Libris Literatuur Prijs van 2018? Het boek gaat over een Turks gezin in de Bijlmer.</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Wees onzichtbaar</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2018: Murat Isik – Wees onzichtbaar</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>!Bijlmermeer flat</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2018: schrijver van 'Wees onzichtbaar'</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Libris Literatuur Prijs van 2018 met de roman 'Wees onzichtbaar'?</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Murat Isik</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2018: Murat Isik – Wees onzichtbaar</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr"/>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>!Bijlmermeer flat</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2019: titel van Rob van Essen</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Rob van Essen de Libris Literatuur Prijs van 2019? Het boek gaat over een vervreemdende nabije toekomst met zelfrijdende auto's.</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>De goede zoon</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2019: Rob van Essen – De goede zoon</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr"/>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>!self-driving car</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2019: schrijver van 'De goede zoon'</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Libris Literatuur Prijs van 2019 met de roman 'De goede zoon'?</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Rob van Essen</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2019: Rob van Essen – De goede zoon</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr"/>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>!self-driving car</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2020: titel van Sander Kollaard</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Sander Kollaard de Libris Literatuur Prijs van 2020? Het boek gaat over een verpleegkundige en zijn hond tijdens een lang weekend.</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Uit het leven van een hond</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2020: Sander Kollaard – Uit het leven van een hond</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr"/>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>!dog walking beach</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2020: schrijver van 'Uit het leven van een hond'</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Libris Literatuur Prijs van 2020 met de roman 'Uit het leven van een hond'?</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Sander Kollaard</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2020: Sander Kollaard – Uit het leven van een hond</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr"/>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>!dog walking beach</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2021: titel van Jeroen Brouwers</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Jeroen Brouwers de Libris Literatuur Prijs van 2021? Het boek gaat over een oude man in een psychiatrische instelling.</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Cliënt E. Busken</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2021: Jeroen Brouwers – Cliënt E. Busken</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr"/>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>!hospital corridor</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2021: schrijver van 'Cliënt E. Busken'</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Libris Literatuur Prijs van 2021 met de roman 'Cliënt E. Busken'?</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Jeroen Brouwers</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2021: Jeroen Brouwers – Cliënt E. Busken</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr"/>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>!hospital corridor</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2022: titel van Mariken Heitman</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Mariken Heitman de Libris Literatuur Prijs van 2022? Het boek gaat over een jonge vrouw die boerin wil worden.</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Wormmaan</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2022: Mariken Heitman – Wormmaan</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr"/>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>!ploughed field soil</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2022: schrijver van 'Wormmaan'</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Libris Literatuur Prijs van 2022 met de roman 'Wormmaan'?</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Mariken Heitman</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2022: Mariken Heitman – Wormmaan</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="inlineStr"/>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>!ploughed field soil</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2023: titel van Anjet Daanje</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Anjet Daanje de Libris Literatuur Prijs van 2023? Het boek gaat over vrouwen door de eeuwen heen, geïnspireerd op Emily Brontë.</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Het lied van ooievaar en dromedaris</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2023: Anjet Daanje – Het lied van ooievaar en dromedaris</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr"/>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>!Yorkshire moors</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2023: schrijver van 'Het lied van ooievaar en dromedaris'</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Libris Literatuur Prijs van 2023 met de roman 'Het lied van ooievaar en dromedaris'?</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Anjet Daanje</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2023: Anjet Daanje – Het lied van ooievaar en dromedaris</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="inlineStr"/>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>!Yorkshire moors</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2024: titel van Rob van Essen</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Rob van Essen de Libris Literatuur Prijs van 2024? Het boek gaat over een man die met een tijdmachine terugreist.</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Ik kom hier nog op terug</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2024: Rob van Essen – Ik kom hier nog op terug</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr"/>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>!vintage radio</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2024: schrijver van 'Ik kom hier nog op terug'</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Libris Literatuur Prijs van 2024 met de roman 'Ik kom hier nog op terug'?</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Rob van Essen</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2024: Rob van Essen – Ik kom hier nog op terug</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="inlineStr"/>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>!vintage radio</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2025: titel van Safae el Khannoussi</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Safae el Khannoussi de Libris Literatuur Prijs van 2025?</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Oroppa</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2025: Safae el Khannoussi – Oroppa</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr"/>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>!Strait of Gibraltar</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2025: schrijver van 'Oroppa'</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Libris Literatuur Prijs van 2025 met de roman 'Oroppa'?</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Safae el Khannoussi</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2025: Safae el Khannoussi – Oroppa</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr"/>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>!Strait of Gibraltar</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2026: titel van Bert Natter</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Bert Natter de Libris Literatuur Prijs van 2026?</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Aan het einde van de oorlog</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2026: Bert Natter – Aan het einde van de oorlog</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr"/>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>!liberation 1945 Netherlands</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2026: schrijver van 'Aan het einde van de oorlog'</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Libris Literatuur Prijs van 2026 met de roman 'Aan het einde van de oorlog'?</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Bert Natter</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Libris Literatuur Prijs 2026: Bert Natter – Aan het einde van de oorlog</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr"/>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>!liberation 1945 Netherlands</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>ECI Literatuurprijs 2016: titel van Martin Michael Driessen</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Martin Michael Driessen de ECI Literatuurprijs van 2016?</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Rivieren</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>ECI Literatuurprijs 2016: Martin Michael Driessen – Rivieren</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr"/>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>!river landscape</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>ECI Literatuurprijs 2016: schrijver van 'Rivieren'</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de ECI Literatuurprijs van 2016 met de roman 'Rivieren'?</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Martin Michael Driessen</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>ECI Literatuurprijs 2016: Martin Michael Driessen – Rivieren</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="inlineStr"/>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>!river landscape</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>ECI Literatuurprijs 2017: titel van Koen Peeters</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Koen Peeters de ECI Literatuurprijs van 2017? Het boek gaat over een traditionele genezer in Congo.</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>De mensengenezer</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>ECI Literatuurprijs 2017: Koen Peeters – De mensengenezer</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr"/>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>!Congo village</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>ECI Literatuurprijs 2017: schrijver van 'De mensengenezer'</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de ECI Literatuurprijs van 2017 met de roman 'De mensengenezer'?</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Koen Peeters</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>ECI Literatuurprijs 2017: Koen Peeters – De mensengenezer</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr"/>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>!Congo village</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>BookSpot Literatuurprijs 2018: titel van Tommy Wieringa</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Tommy Wieringa de BookSpot Literatuurprijs van 2018? Het boek gaat over een man in een Twents grensdorp.</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>De heilige Rita</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>BookSpot Literatuurprijs 2018: Tommy Wieringa – De heilige Rita</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr"/>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>!Twente landscape</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>BookSpot Literatuurprijs 2018: schrijver van 'De heilige Rita'</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de BookSpot Literatuurprijs van 2018 met de roman 'De heilige Rita'?</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Tommy Wieringa</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>BookSpot Literatuurprijs 2018: Tommy Wieringa – De heilige Rita</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr"/>
+      <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>!Twente landscape</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>BookSpot Literatuurprijs 2019: titel van Wessel te Gussinklo</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Wessel te Gussinklo de BookSpot Literatuurprijs van 2019? Het boek gaat over een puber op zomerkamp.</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>De hoogstapelaar</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>BookSpot Literatuurprijs 2019: Wessel te Gussinklo – De hoogstapelaar</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr"/>
+      <c r="G52" s="8" t="inlineStr">
+        <is>
+          <t>!summer camp tents</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>BookSpot Literatuurprijs 2019: schrijver van 'De hoogstapelaar'</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de BookSpot Literatuurprijs van 2019 met de roman 'De hoogstapelaar'?</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Wessel te Gussinklo</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>BookSpot Literatuurprijs 2019: Wessel te Gussinklo – De hoogstapelaar</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr"/>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>!summer camp tents</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2020: titel van Oek de Jong</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Oek de Jong de Boekenbon Literatuurprijs van 2020? Het boek gaat over een kunstschilder die achtervolgd wordt door een jeugddrama met brand.</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Zwarte schuur</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2020: Oek de Jong – Zwarte schuur</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="inlineStr"/>
+      <c r="G54" s="8" t="inlineStr">
+        <is>
+          <t>!barn fire</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2020: schrijver van 'Zwarte schuur'</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Boekenbon Literatuurprijs van 2020 met de roman 'Zwarte schuur'?</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Oek de Jong</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2020: Oek de Jong – Zwarte schuur</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr"/>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>!barn fire</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2021: titel van Wessel te Gussinklo</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Wessel te Gussinklo de Boekenbon Literatuurprijs van 2021?</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Op weg naar de Hartz</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2021: Wessel te Gussinklo – Op weg naar de Hartz</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="inlineStr"/>
+      <c r="G56" s="8" t="inlineStr">
+        <is>
+          <t>!German forest mountains</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2021: schrijver van 'Op weg naar de Hartz'</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Boekenbon Literatuurprijs van 2021 met de roman 'Op weg naar de Hartz'?</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Wessel te Gussinklo</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2021: Wessel te Gussinklo – Op weg naar de Hartz</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="inlineStr"/>
+      <c r="G57" s="8" t="inlineStr">
+        <is>
+          <t>!German forest mountains</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2022: titel van Anjet Daanje</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Anjet Daanje de Boekenbon Literatuurprijs van 2022?</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Het lied van ooievaar en dromedaris</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2022: Anjet Daanje – Het lied van ooievaar en dromedaris</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="inlineStr"/>
+      <c r="G58" s="8" t="inlineStr">
+        <is>
+          <t>!Haworth moor</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2022: schrijver van 'Het lied van ooievaar en dromedaris'</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Boekenbon Literatuurprijs van 2022 met de roman 'Het lied van ooievaar en dromedaris'?</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Anjet Daanje</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2022: Anjet Daanje – Het lied van ooievaar en dromedaris</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="inlineStr"/>
+      <c r="G59" s="8" t="inlineStr">
+        <is>
+          <t>!Haworth moor</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2023: titel van Jan Vantoortelboom</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Jan Vantoortelboom de Boekenbon Literatuurprijs van 2023?</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Mauk</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2023: Jan Vantoortelboom – Mauk</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="inlineStr"/>
+      <c r="G60" s="8" t="inlineStr">
+        <is>
+          <t>!Flemish village</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2023: schrijver van 'Mauk'</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Boekenbon Literatuurprijs van 2023 met de roman 'Mauk'?</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Jan Vantoortelboom</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2023: Jan Vantoortelboom – Mauk</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="inlineStr"/>
+      <c r="G61" s="8" t="inlineStr">
+        <is>
+          <t>!Flemish village</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2024: titel van Esther Gerritsen</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Esther Gerritsen de Boekenbon Literatuurprijs van 2024?</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Gebied 19</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2024: Esther Gerritsen – Gebied 19</t>
+        </is>
+      </c>
+      <c r="F62" s="9" t="inlineStr"/>
+      <c r="G62" s="8" t="inlineStr">
+        <is>
+          <t>!abstract painting</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2024: schrijver van 'Gebied 19'</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Boekenbon Literatuurprijs van 2024 met de roman 'Gebied 19'?</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Esther Gerritsen</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2024: Esther Gerritsen – Gebied 19</t>
+        </is>
+      </c>
+      <c r="F63" s="9" t="inlineStr"/>
+      <c r="G63" s="8" t="inlineStr">
+        <is>
+          <t>!abstract painting</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2025: titel van Charlotte Van den Broeck</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Met welke roman won Charlotte Van den Broeck de Boekenbon Literatuurprijs van 2025?</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Een vlam Tasmaanse tijgers</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2025: Charlotte Van den Broeck – Een vlam Tasmaanse tijgers</t>
+        </is>
+      </c>
+      <c r="F64" s="9" t="inlineStr"/>
+      <c r="G64" s="8" t="inlineStr">
+        <is>
+          <t>!natural history museum</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2025: schrijver van 'Een vlam Tasmaanse tijgers'</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Wie won de Boekenbon Literatuurprijs van 2025 met de roman 'Een vlam Tasmaanse tijgers'?</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Charlotte Van den Broeck</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>Boekenbon Literatuurprijs 2025: Charlotte Van den Broeck – Een vlam Tasmaanse tijgers</t>
+        </is>
+      </c>
+      <c r="F65" s="9" t="inlineStr"/>
+      <c r="G65" s="8" t="inlineStr">
+        <is>
+          <t>!natural history museum</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Literatuurprijzen: uitgebreide plotbeschrijving in de vragen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GWDzH9CBKYVCbFWmsbqcR
</commit_message>
<xml_diff>
--- a/stamlijsten.xlsx
+++ b/stamlijsten.xlsx
@@ -5962,7 +5962,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Connie Palmen de Libris Literatuur Prijs van 2016? Het boek gaat over het huwelijk van Ted Hughes en Sylvia Plath.</t>
+          <t>In deze roman kijkt de Engelse dichter Ted Hughes terug op zijn stormachtige huwelijk met de Amerikaanse dichteres Sylvia Plath, die in 1963 zelfmoord pleegde. Hij verdedigt zich tegen de beschuldiging dat hij haar dood op zijn geweten heeft. Met welk boek won Connie Palmen hiermee de Libris Literatuur Prijs van 2016?</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
@@ -5994,7 +5994,7 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Libris Literatuur Prijs van 2016 met de roman 'Jij zegt het'?</t>
+          <t>In deze roman kijkt de Engelse dichter Ted Hughes terug op zijn stormachtige huwelijk met de Amerikaanse dichteres Sylvia Plath, die in 1963 zelfmoord pleegde. Hij verdedigt zich tegen de beschuldiging dat hij haar dood op zijn geweten heeft. Wie won met de roman 'Jij zegt het' de Libris Literatuur Prijs van 2016?</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr">
@@ -6026,7 +6026,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Alfred Birney de Libris Literatuur Prijs van 2017? Het boek gaat over een Indische vader en de koloniale oorlog.</t>
+          <t>Een zoon reconstrueert het leven van zijn Indische vader, die tijdens de Indonesische onafhankelijkheidsoorlog als vertaler en vechter gruweldaden beging en later in Nederland zijn gezin terroriseerde. Met welk boek won Alfred Birney hiermee de Libris Literatuur Prijs van 2017?</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
@@ -6042,7 +6042,7 @@
       <c r="F26" s="9" t="inlineStr"/>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>!Java rice field</t>
+          <t>!Indonesia rice terraces</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr"/>
@@ -6058,7 +6058,7 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Libris Literatuur Prijs van 2017 met de roman 'De tolk van Java'?</t>
+          <t>Een zoon reconstrueert het leven van zijn Indische vader, die tijdens de Indonesische onafhankelijkheidsoorlog als vertaler en vechter gruweldaden beging en later in Nederland zijn gezin terroriseerde. Wie won met de roman 'De tolk van Java' de Libris Literatuur Prijs van 2017?</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr">
@@ -6074,7 +6074,7 @@
       <c r="F27" s="9" t="inlineStr"/>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>!Java rice field</t>
+          <t>!Indonesia rice terraces</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr"/>
@@ -6090,7 +6090,7 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Murat Isik de Libris Literatuur Prijs van 2018? Het boek gaat over een Turks gezin in de Bijlmer.</t>
+          <t>De jonge Metin groeit op in een Turks gezin dat in de jaren tachtig in de Amsterdamse Bijlmer belandt. Zijn vader is gewelddadig, en Metin probeert zich met boeken en tekenen een weg naar een ander leven te banen. Met welk boek won Murat Isik hiermee de Libris Literatuur Prijs van 2018?</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -6122,7 +6122,7 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Libris Literatuur Prijs van 2018 met de roman 'Wees onzichtbaar'?</t>
+          <t>De jonge Metin groeit op in een Turks gezin dat in de jaren tachtig in de Amsterdamse Bijlmer belandt. Zijn vader is gewelddadig, en Metin probeert zich met boeken en tekenen een weg naar een ander leven te banen. Wie won met de roman 'Wees onzichtbaar' de Libris Literatuur Prijs van 2018?</t>
         </is>
       </c>
       <c r="D29" s="8" t="inlineStr">
@@ -6154,7 +6154,7 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Rob van Essen de Libris Literatuur Prijs van 2019? Het boek gaat over een vervreemdende nabije toekomst met zelfrijdende auto's.</t>
+          <t>Een zestigjarige man rijdt door een nabije toekomst vol pratende, zelfrijdende auto's en haalt herinneringen op aan zijn net overleden, demente moeder. Een absurde sciencefictionroman vol bizarre humor. Met welk boek won Rob van Essen hiermee de Libris Literatuur Prijs van 2019?</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -6186,7 +6186,7 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Libris Literatuur Prijs van 2019 met de roman 'De goede zoon'?</t>
+          <t>Een zestigjarige man rijdt door een nabije toekomst vol pratende, zelfrijdende auto's en haalt herinneringen op aan zijn net overleden, demente moeder. Een absurde sciencefictionroman vol bizarre humor. Wie won met de roman 'De goede zoon' de Libris Literatuur Prijs van 2019?</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -6218,7 +6218,7 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Sander Kollaard de Libris Literatuur Prijs van 2020? Het boek gaat over een verpleegkundige en zijn hond tijdens een lang weekend.</t>
+          <t>We volgen Henk, een vijftigjarige verpleegkundige, gedurende een lang weekend met zijn trouwe huisdier. Er gebeurt weinig, maar in kleine voorvallen komen liefde, ouder worden en sterfelijkheid voorbij. Met welk boek won Sander Kollaard hiermee de Libris Literatuur Prijs van 2020?</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
@@ -6250,7 +6250,7 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Libris Literatuur Prijs van 2020 met de roman 'Uit het leven van een hond'?</t>
+          <t>We volgen Henk, een vijftigjarige verpleegkundige, gedurende een lang weekend met zijn trouwe huisdier. Er gebeurt weinig, maar in kleine voorvallen komen liefde, ouder worden en sterfelijkheid voorbij. Wie won met de roman 'Uit het leven van een hond' de Libris Literatuur Prijs van 2020?</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Jeroen Brouwers de Libris Literatuur Prijs van 2021? Het boek gaat over een oude man in een psychiatrische instelling.</t>
+          <t>Een oude man zit opgesloten in een psychiatrische instelling. Hij voelt zich vernederd en vervolgd door het personeel en verzet zich met woede en zwarte humor tegen zijn aftakeling. Met welk boek won Jeroen Brouwers hiermee de Libris Literatuur Prijs van 2021?</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Libris Literatuur Prijs van 2021 met de roman 'Cliënt E. Busken'?</t>
+          <t>Een oude man zit opgesloten in een psychiatrische instelling. Hij voelt zich vernederd en vervolgd door het personeel en verzet zich met woede en zwarte humor tegen zijn aftakeling. Wie won met de roman 'Cliënt E. Busken' de Libris Literatuur Prijs van 2021?</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Mariken Heitman de Libris Literatuur Prijs van 2022? Het boek gaat over een jonge vrouw die boerin wil worden.</t>
+          <t>Een jonge vrouw keert de stad de rug toe en wil met haar handen in de grond werken. Ze leert het boerenvak op akkers en in tuinen, en zoekt haar plek tussen natuur, werk en eenzaamheid. Met welk boek won Mariken Heitman hiermee de Libris Literatuur Prijs van 2022?</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -6378,7 +6378,7 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Libris Literatuur Prijs van 2022 met de roman 'Wormmaan'?</t>
+          <t>Een jonge vrouw keert de stad de rug toe en wil met haar handen in de grond werken. Ze leert het boerenvak op akkers en in tuinen, en zoekt haar plek tussen natuur, werk en eenzaamheid. Wie won met de roman 'Wormmaan' de Libris Literatuur Prijs van 2022?</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
@@ -6410,7 +6410,7 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Anjet Daanje de Libris Literatuur Prijs van 2023? Het boek gaat over vrouwen door de eeuwen heen, geïnspireerd op Emily Brontë.</t>
+          <t>Vrouwen uit verschillende eeuwen zijn elk op hun eigen manier verbonden met een negentiende-eeuwse schrijfster, gemodelleerd naar Emily Brontë. Samen vormen hun verhalen een portret van haar nagelaten leven. Met welk boek won Anjet Daanje hiermee de Libris Literatuur Prijs van 2023?</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
@@ -6442,7 +6442,7 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Libris Literatuur Prijs van 2023 met de roman 'Het lied van ooievaar en dromedaris'?</t>
+          <t>Vrouwen uit verschillende eeuwen zijn elk op hun eigen manier verbonden met een negentiende-eeuwse schrijfster, gemodelleerd naar Emily Brontë. Samen vormen hun verhalen een portret van haar nagelaten leven. Wie won met de roman 'Het lied van ooievaar en dromedaris' de Libris Literatuur Prijs van 2023?</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Rob van Essen de Libris Literatuur Prijs van 2024? Het boek gaat over een man die met een tijdmachine terugreist.</t>
+          <t>Een man van in de zestig krijgt van een oude studievriend uit Los Angeles de kans om naar het verleden te reizen. Hij belandt in het Amsterdam van de late jaren tachtig, waar ook zijn oude vrienden blijken te zitten, en ze kunnen er niet meer weg. Met welk boek won Rob van Essen hiermee de Libris Literatuur Prijs van 2024?</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
@@ -6510,7 +6510,7 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Libris Literatuur Prijs van 2024 met de roman 'Ik kom hier nog op terug'?</t>
+          <t>Een man van in de zestig krijgt van een oude studievriend uit Los Angeles de kans om naar het verleden te reizen. Hij belandt in het Amsterdam van de late jaren tachtig, waar ook zijn oude vrienden blijken te zitten, en ze kunnen er niet meer weg. Wie won met de roman 'Ik kom hier nog op terug' de Libris Literatuur Prijs van 2024?</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
@@ -6546,7 +6546,7 @@
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Safae el Khannoussi de Libris Literatuur Prijs van 2025?</t>
+          <t>Een Joods-Marokkaanse kunstenares verdwijnt op het hoogtepunt van haar carrière. Haar verdwijning brengt migranten en buitenstaanders in Amsterdam, Parijs en Casablanca samen, en legt de verborgen geschiedenis van de politieke onderdrukking in Marokko bloot. Met welk boek won Safae el Khannoussi hiermee de Libris Literatuur Prijs van 2025?</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
@@ -6582,7 +6582,7 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Libris Literatuur Prijs van 2025 met de roman 'Oroppa'?</t>
+          <t>Een Joods-Marokkaanse kunstenares verdwijnt op het hoogtepunt van haar carrière. Haar verdwijning brengt migranten en buitenstaanders in Amsterdam, Parijs en Casablanca samen, en legt de verborgen geschiedenis van de politieke onderdrukking in Marokko bloot. Wie won met de roman 'Oroppa' de Libris Literatuur Prijs van 2025?</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
@@ -6618,7 +6618,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Bert Natter de Libris Literatuur Prijs van 2026?</t>
+          <t>Op 20 april 1945, terwijl het Rode Leger nadert, raakt het elfjarige zoontje van de plaatsvervangend commandant van een concentratiekamp bij Berlijn vermist bij een meer. In ruim twintig uur volgen we daders en gevangenen in de laatste dagen van het kamp. Met welk boek won Bert Natter hiermee de Libris Literatuur Prijs van 2026?</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
@@ -6634,7 +6634,7 @@
       <c r="F44" s="9" t="inlineStr"/>
       <c r="G44" s="8" t="inlineStr">
         <is>
-          <t>!liberation 1945 Netherlands</t>
+          <t>!lake forest Brandenburg</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr"/>
@@ -6650,7 +6650,7 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Libris Literatuur Prijs van 2026 met de roman 'Aan het einde van de oorlog'?</t>
+          <t>Op 20 april 1945, terwijl het Rode Leger nadert, raakt het elfjarige zoontje van de plaatsvervangend commandant van een concentratiekamp bij Berlijn vermist bij een meer. In ruim twintig uur volgen we daders en gevangenen in de laatste dagen van het kamp. Wie won met de roman 'Aan het einde van de oorlog' de Libris Literatuur Prijs van 2026?</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
@@ -6666,7 +6666,7 @@
       <c r="F45" s="9" t="inlineStr"/>
       <c r="G45" s="8" t="inlineStr">
         <is>
-          <t>!liberation 1945 Netherlands</t>
+          <t>!lake forest Brandenburg</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr"/>
@@ -6682,7 +6682,7 @@
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Martin Michael Driessen de ECI Literatuurprijs van 2016?</t>
+          <t>Drie novellen, elk rond stromend water: een acteur met een drankprobleem maakt een kanotocht door de Ardennen die uitloopt op een hellevaart, twee houtvlotters leven langs de Main en de Rijn, en een beek in Bretagne scheidt twee vijandige families. Met welk boek won Martin Michael Driessen hiermee de ECI Literatuurprijs van 2016?</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
@@ -6698,7 +6698,7 @@
       <c r="F46" s="9" t="inlineStr"/>
       <c r="G46" s="8" t="inlineStr">
         <is>
-          <t>!river landscape</t>
+          <t>!Ardennes canoe</t>
         </is>
       </c>
       <c r="H46" s="6" t="inlineStr"/>
@@ -6714,7 +6714,7 @@
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Wie won de ECI Literatuurprijs van 2016 met de roman 'Rivieren'?</t>
+          <t>Drie novellen, elk rond stromend water: een acteur met een drankprobleem maakt een kanotocht door de Ardennen die uitloopt op een hellevaart, twee houtvlotters leven langs de Main en de Rijn, en een beek in Bretagne scheidt twee vijandige families. Wie won met de roman 'Rivieren' de ECI Literatuurprijs van 2016?</t>
         </is>
       </c>
       <c r="D47" s="8" t="inlineStr">
@@ -6730,7 +6730,7 @@
       <c r="F47" s="9" t="inlineStr"/>
       <c r="G47" s="8" t="inlineStr">
         <is>
-          <t>!river landscape</t>
+          <t>!Ardennes canoe</t>
         </is>
       </c>
       <c r="H47" s="6" t="inlineStr"/>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Koen Peeters de ECI Literatuurprijs van 2017? Het boek gaat over een traditionele genezer in Congo.</t>
+          <t>Een boerenzoon uit de Westhoek ontvlucht het platteland door priester en missionaris te worden. In Congo ontdekt hij wie hij werkelijk is en vindt hij zijn talent om mensen te helpen en te genezen. Losjes gebaseerd op het leven van antropoloog Renaat Devisch. Met welk boek won Koen Peeters hiermee de ECI Literatuurprijs van 2017?</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
@@ -6778,7 +6778,7 @@
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Wie won de ECI Literatuurprijs van 2017 met de roman 'De mensengenezer'?</t>
+          <t>Een boerenzoon uit de Westhoek ontvlucht het platteland door priester en missionaris te worden. In Congo ontdekt hij wie hij werkelijk is en vindt hij zijn talent om mensen te helpen en te genezen. Losjes gebaseerd op het leven van antropoloog Renaat Devisch. Wie won met de roman 'De mensengenezer' de ECI Literatuurprijs van 2017?</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
@@ -6810,7 +6810,7 @@
       </c>
       <c r="C50" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Tommy Wieringa de BookSpot Literatuurprijs van 2018? Het boek gaat over een man in een Twents grensdorp.</t>
+          <t>Een eenzame vijftiger woont in een Twents dorp aan de Duitse grens. Als kind verloor hij zijn vader toen een Russisch vliegtuigje in het dorp neerstortte, en sindsdien leeft hij tussen zijn handel in oude spullen en een paar gesprekken met een jeugdvriend. Met welk boek won Tommy Wieringa hiermee de BookSpot Literatuurprijs van 2018?</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
@@ -6842,7 +6842,7 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Wie won de BookSpot Literatuurprijs van 2018 met de roman 'De heilige Rita'?</t>
+          <t>Een eenzame vijftiger woont in een Twents dorp aan de Duitse grens. Als kind verloor hij zijn vader toen een Russisch vliegtuigje in het dorp neerstortte, en sindsdien leeft hij tussen zijn handel in oude spullen en een paar gesprekken met een jeugdvriend. Wie won met de roman 'De heilige Rita' de BookSpot Literatuurprijs van 2018?</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
@@ -6874,7 +6874,7 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Wessel te Gussinklo de BookSpot Literatuurprijs van 2019? Het boek gaat over een puber op zomerkamp.</t>
+          <t>De bijna achttienjarige Ewout Meyster, van kostschool gestuurd, wil zijn naïeve vrienden imponeren met zijn superioriteit en oefent voor de spiegel hoe hij een echte persoonlijkheid wordt, terwijl hij geplaagd wordt door angsten en depressies. Met welk boek won Wessel te Gussinklo hiermee de BookSpot Literatuurprijs van 2019?</t>
         </is>
       </c>
       <c r="D52" s="8" t="inlineStr">
@@ -6890,7 +6890,7 @@
       <c r="F52" s="9" t="inlineStr"/>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t>!summer camp tents</t>
+          <t>!mirror young man shadow</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr"/>
@@ -6906,7 +6906,7 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Wie won de BookSpot Literatuurprijs van 2019 met de roman 'De hoogstapelaar'?</t>
+          <t>De bijna achttienjarige Ewout Meyster, van kostschool gestuurd, wil zijn naïeve vrienden imponeren met zijn superioriteit en oefent voor de spiegel hoe hij een echte persoonlijkheid wordt, terwijl hij geplaagd wordt door angsten en depressies. Wie won met de roman 'De hoogstapelaar' de BookSpot Literatuurprijs van 2019?</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
@@ -6922,7 +6922,7 @@
       <c r="F53" s="9" t="inlineStr"/>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t>!summer camp tents</t>
+          <t>!mirror young man shadow</t>
         </is>
       </c>
       <c r="H53" s="6" t="inlineStr"/>
@@ -6938,7 +6938,7 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Oek de Jong de Boekenbon Literatuurprijs van 2020? Het boek gaat over een kunstschilder die achtervolgd wordt door een jeugddrama met brand.</t>
+          <t>Een succesvolle kunstschilder wordt achtervolgd door een gebeurtenis uit zijn jeugd in Zeeland: een brand waarbij een meisje omkwam en waarvoor hij zich schuldig voelt. Met welk boek won Oek de Jong hiermee de Boekenbon Literatuurprijs van 2020?</t>
         </is>
       </c>
       <c r="D54" s="8" t="inlineStr">
@@ -6954,7 +6954,7 @@
       <c r="F54" s="9" t="inlineStr"/>
       <c r="G54" s="8" t="inlineStr">
         <is>
-          <t>!barn fire</t>
+          <t>!Zeeland polder</t>
         </is>
       </c>
       <c r="H54" s="6" t="inlineStr"/>
@@ -6970,7 +6970,7 @@
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Boekenbon Literatuurprijs van 2020 met de roman 'Zwarte schuur'?</t>
+          <t>Een succesvolle kunstschilder wordt achtervolgd door een gebeurtenis uit zijn jeugd in Zeeland: een brand waarbij een meisje omkwam en waarvoor hij zich schuldig voelt. Wie won met de roman 'Zwarte schuur' de Boekenbon Literatuurprijs van 2020?</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
@@ -6986,7 +6986,7 @@
       <c r="F55" s="9" t="inlineStr"/>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>!barn fire</t>
+          <t>!Zeeland polder</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr"/>
@@ -7002,7 +7002,7 @@
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Wessel te Gussinklo de Boekenbon Literatuurprijs van 2021?</t>
+          <t>Een angstige, gespannen man reist naar het landgoed van "de Grote Man", die er een hogeschool leidt, om zich bij een groep docenten aan te sluiten. Onderweg loopt alles uit de hand door zijn eigen achterdocht. Het is de tweede prijs van de schrijver, na 2019. Met welk boek won Wessel te Gussinklo hiermee de Boekenbon Literatuurprijs van 2021?</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
@@ -7018,7 +7018,7 @@
       <c r="F56" s="9" t="inlineStr"/>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>!German forest mountains</t>
+          <t>!country estate manor</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr"/>
@@ -7034,7 +7034,7 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Boekenbon Literatuurprijs van 2021 met de roman 'Op weg naar de Hartz'?</t>
+          <t>Een angstige, gespannen man reist naar het landgoed van "de Grote Man", die er een hogeschool leidt, om zich bij een groep docenten aan te sluiten. Onderweg loopt alles uit de hand door zijn eigen achterdocht. Het is de tweede prijs van de schrijver, na 2019. Wie won met de roman 'Op weg naar de Hartz' de Boekenbon Literatuurprijs van 2021?</t>
         </is>
       </c>
       <c r="D57" s="8" t="inlineStr">
@@ -7050,7 +7050,7 @@
       <c r="F57" s="9" t="inlineStr"/>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>!German forest mountains</t>
+          <t>!country estate manor</t>
         </is>
       </c>
       <c r="H57" s="6" t="inlineStr"/>
@@ -7066,7 +7066,7 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Anjet Daanje de Boekenbon Literatuurprijs van 2022?</t>
+          <t>Vrouwen uit verschillende eeuwen zijn elk op hun eigen manier verbonden met een negentiende-eeuwse schrijfster, gemodelleerd naar Emily Brontë. Dit boek won ook de Libris van 2023. Met welk boek won Anjet Daanje hiermee de Boekenbon Literatuurprijs van 2022?</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
@@ -7098,7 +7098,7 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Boekenbon Literatuurprijs van 2022 met de roman 'Het lied van ooievaar en dromedaris'?</t>
+          <t>Vrouwen uit verschillende eeuwen zijn elk op hun eigen manier verbonden met een negentiende-eeuwse schrijfster, gemodelleerd naar Emily Brontë. Dit boek won ook de Libris van 2023. Wie won met de roman 'Het lied van ooievaar en dromedaris' de Boekenbon Literatuurprijs van 2022?</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
@@ -7130,7 +7130,7 @@
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Jan Vantoortelboom de Boekenbon Literatuurprijs van 2023?</t>
+          <t>Een man van in de zeventig ligt op sterven en blikt terug op zijn traumatische jeugd met een gewelddadige vader. Hij overleefde dankzij zijn verbeelding en zijn steun Henri, de oudere broer die hij altijd had gewild. Met welk boek won Jan Vantoortelboom hiermee de Boekenbon Literatuurprijs van 2023?</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
@@ -7162,7 +7162,7 @@
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Boekenbon Literatuurprijs van 2023 met de roman 'Mauk'?</t>
+          <t>Een man van in de zeventig ligt op sterven en blikt terug op zijn traumatische jeugd met een gewelddadige vader. Hij overleefde dankzij zijn verbeelding en zijn steun Henri, de oudere broer die hij altijd had gewild. Wie won met de roman 'Mauk' de Boekenbon Literatuurprijs van 2023?</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
@@ -7194,7 +7194,7 @@
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Esther Gerritsen de Boekenbon Literatuurprijs van 2024?</t>
+          <t>Speculatieve roman: de helft van de mensheid vertrekt naar een andere planeet, waar mensen zonder pijnlijke herinneringen leven dankzij een ingreep in de hersenen. Tomas Boom blijft met zijn hond achter in een Nederlands dorp, nadat zijn vrouw en zoontje plotseling verdwenen zijn. Met welk boek won Esther Gerritsen hiermee de Boekenbon Literatuurprijs van 2024?</t>
         </is>
       </c>
       <c r="D62" s="8" t="inlineStr">
@@ -7210,7 +7210,7 @@
       <c r="F62" s="9" t="inlineStr"/>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>!abstract painting</t>
+          <t>!exoplanet night sky</t>
         </is>
       </c>
       <c r="H62" s="6" t="inlineStr"/>
@@ -7226,7 +7226,7 @@
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Boekenbon Literatuurprijs van 2024 met de roman 'Gebied 19'?</t>
+          <t>Speculatieve roman: de helft van de mensheid vertrekt naar een andere planeet, waar mensen zonder pijnlijke herinneringen leven dankzij een ingreep in de hersenen. Tomas Boom blijft met zijn hond achter in een Nederlands dorp, nadat zijn vrouw en zoontje plotseling verdwenen zijn. Wie won met de roman 'Gebied 19' de Boekenbon Literatuurprijs van 2024?</t>
         </is>
       </c>
       <c r="D63" s="8" t="inlineStr">
@@ -7242,7 +7242,7 @@
       <c r="F63" s="9" t="inlineStr"/>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>!abstract painting</t>
+          <t>!exoplanet night sky</t>
         </is>
       </c>
       <c r="H63" s="6" t="inlineStr"/>
@@ -7258,7 +7258,7 @@
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>Met welke roman won Charlotte Van den Broeck de Boekenbon Literatuurprijs van 2025?</t>
+          <t>Verhalende non-fictie: de schrijfster volgt het spoor van een uitgestorven buideldier en denkt na over verlies, hoop in tijden van klimaatcrisis en de kracht van verhalen. Met welk boek won Charlotte Van den Broeck hiermee de Boekenbon Literatuurprijs van 2025?</t>
         </is>
       </c>
       <c r="D64" s="8" t="inlineStr">
@@ -7290,7 +7290,7 @@
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>Wie won de Boekenbon Literatuurprijs van 2025 met de roman 'Een vlam Tasmaanse tijgers'?</t>
+          <t>Verhalende non-fictie: de schrijfster volgt het spoor van een uitgestorven buideldier en denkt na over verlies, hoop in tijden van klimaatcrisis en de kracht van verhalen. Wie won met het boek 'Een vlam Tasmaanse tijgers' de Boekenbon Literatuurprijs van 2025?</t>
         </is>
       </c>
       <c r="D65" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Literatuurprijzen: werkbeschrijving met titels bij Nobel- en P.C. Hooft-kaarten
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GWDzH9CBKYVCbFWmsbqcR
</commit_message>
<xml_diff>
--- a/stamlijsten.xlsx
+++ b/stamlijsten.xlsx
@@ -5258,7 +5258,7 @@
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>De Nobelprijs voor de Literatuur van 2016 ging naar een Amerikaanse singer-songwriter, als eerste musicus. Wie is dit?</t>
+          <t>Deze Amerikaanse singer-songwriter schreef liedjes als 'Blowin' in the Wind', 'The Times They Are a-Changin'' en 'Like a Rolling Stone'. Hij was de eerste musicus die de prijs kreeg en kwam hem niet persoonlijk ophalen. Wie kreeg de Nobelprijs voor de Literatuur van 2016?</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
@@ -5290,7 +5290,7 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>De Nobelprijs voor de Literatuur van 2017 ging naar een Britse romanschrijver die in Japan werd geboren. Wie is dit?</t>
+          <t>Deze Britse schrijver, geboren in Nagasaki, schreef 'The Remains of the Day', over een butler die terugkijkt op zijn leven in dienst van een lord (verfilmd met Anthony Hopkins), en 'Never Let Me Go', over kinderen op een kostschool die gekloond blijken te zijn. Wie kreeg de Nobelprijs voor de Literatuur van 2017?</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
@@ -5322,7 +5322,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>De Nobelprijs voor de Literatuur van 2018 ging naar een Poolse schrijfster; haar prijs werd een jaar later uitgereikt. Wie is dit?</t>
+          <t>Deze Poolse schrijfster schreef 'Jaag je ploeg over de botten der doden', over een oudere vrouw die in een berggebied raadselachtige sterfgevallen onderzoekt, en het lijvige 'De jakobsboeken'. Haar prijs werd een jaar later uitgereikt, na een schandaal bij de Zweedse Academie. Wie kreeg de Nobelprijs voor de Literatuur van 2018?</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
@@ -5354,7 +5354,7 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>De Nobelprijs voor de Literatuur van 2019 ging naar een Oostenrijkse schrijver en toneelauteur. Wie is dit?</t>
+          <t>Deze Oostenrijkse schrijver schreef 'De angst van de doelman voor de strafschop' en het scenario van Wim Wenders' film 'Der Himmel über Berlin'. De toekenning was omstreden door zijn steun aan de Servische leider Milošević. Wie kreeg de Nobelprijs voor de Literatuur van 2019?</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
@@ -5386,7 +5386,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>De Nobelprijs voor de Literatuur van 2020 ging naar een Amerikaanse dichteres. Wie is dit?</t>
+          <t>Deze Amerikaanse dichteres won de Pulitzerprijs met de bundel 'The Wild Iris', waarin bloemen in een tuin het woord voeren. Ook 'Averno' is een bekende bundel van haar. Wie kreeg de Nobelprijs voor de Literatuur van 2020?</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
@@ -5418,7 +5418,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>De Nobelprijs voor de Literatuur van 2021 ging naar een schrijver die op Zanzibar werd geboren en in Engeland woont. Wie is dit?</t>
+          <t>Deze schrijver, geboren op Zanzibar en woonachtig in Engeland, schreef 'Paradise', over een jongen die door zijn vader aan een koopman wordt verpand in koloniaal Oost-Afrika, en 'Afterlives'. Hij schrijft over kolonialisme en vluchtelingen. Wie kreeg de Nobelprijs voor de Literatuur van 2021?</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -5450,7 +5450,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>De Nobelprijs voor de Literatuur van 2022 ging naar een Franse schrijfster van autobiografisch werk. Wie is dit?</t>
+          <t>Deze Franse schrijfster schreef autobiografisch werk als 'De jaren', een collectieve biografie van haar generatie, en 'Het voorval', over haar illegale abortus in 1963. Wie kreeg de Nobelprijs voor de Literatuur van 2022?</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -5482,7 +5482,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>De Nobelprijs voor de Literatuur van 2023 ging naar een Noorse toneelschrijver en romancier. Wie is dit?</t>
+          <t>Deze Noorse toneelschrijver en romancier schreef de zevendelige roman 'Septologie', geschreven in één lange zin, en het toneelstuk 'Iemand komt'. Hij is na Ibsen de meest gespeelde Noorse toneelschrijver. Wie kreeg de Nobelprijs voor de Literatuur van 2023?</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>De Nobelprijs voor de Literatuur van 2024 ging naar een Zuid-Koreaanse schrijfster, als eerste Aziatische vrouw. Wie is dit?</t>
+          <t>Deze Zuid-Koreaanse schrijfster schreef 'De vegetariër', over een vrouw die weigert nog vlees te eten, en 'Mensenwerk', over het bloedig neergeslagen studentenprotest in Gwangju in 1980. Ze was de eerste Aziatische vrouw met deze prijs. Wie kreeg de Nobelprijs voor de Literatuur van 2024?</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>De Nobelprijs voor de Literatuur van 2025 ging naar een Hongaarse schrijver van lange, apocalyptische romans. Wie is dit?</t>
+          <t>Deze Hongaarse schrijver staat bekend om zinnen die pagina's lang doorlopen. Zijn roman 'Satanstango', over een vervallen dorpscollectief, werd door Béla Tarr verfilmd tot een film van zeven uur. Wie kreeg de Nobelprijs voor de Literatuur van 2025?</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
@@ -5578,7 +5578,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>De Nobelprijs voor de Literatuur van 2026 ging naar een Canadese dichteres en classica. Wie is dit?</t>
+          <t>Deze Canadese dichteres en classica schreef 'Autobiography of Red', een roman in verzen over een Grieks mythologisch monster, en vertaalde Sappho. Ze werkt vaak met Griekse klassiekers. Wie kreeg de Nobelprijs voor de Literatuur van 2026?</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
@@ -5610,7 +5610,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>De P.C. Hooft-prijs van 2016, voor verhalend proza, ging naar een Surinaams-Nederlandse schrijfster. Wie is dit?</t>
+          <t>Deze Surinaams-Nederlandse schrijfster schreef 'Over de gekte van een vrouw' en de trilogie 'Gewaagd leven', 'Was getekend' en 'Lijken op liefde' over Suriname. Ze was de eerste Surinaamse winnaar. Wie kreeg de P.C. Hooft-prijs van 2016, voor verhalend proza?</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -5642,7 +5642,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>De P.C. Hooft-prijs van 2017, voor beschouwend proza, ging naar een essayist en NRC-columnist. Wie is dit?</t>
+          <t>Deze essayist en NRC-columnist schreef het essay 'Onbehagen', over het nieuwe Nederland, en schrijft over identiteit en de tijdgeest. Wie kreeg de P.C. Hooft-prijs van 2017, voor beschouwend proza?</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -5674,7 +5674,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>De P.C. Hooft-prijs van 2018, voor poëzie, ging naar een dichter en hoogleraar economie. Wie is dit?</t>
+          <t>Deze dichter is ook hoogleraar economie. Hij schrijft verhalende, ironische gedichten, vaak over macht en geld. Wie kreeg de P.C. Hooft-prijs van 2018, voor poëzie?</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
@@ -5706,7 +5706,7 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>De P.C. Hooft-prijs van 2019, voor verhalend proza, ging naar een schrijfster van Het bittere kruid. Wie is dit?</t>
+          <t>Deze schrijfster werd bekend met 'Het bittere kruid' (1957), over een Joods meisje dat in de oorlog als enige van haar familie overleeft. Ook 'Een leeg huis' en 'De glazen brug' zijn van haar. Wie kreeg de P.C. Hooft-prijs van 2019, voor verhalend proza?</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -5738,7 +5738,7 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>De P.C. Hooft-prijs van 2020, voor beschouwend proza, ging naar een filosoof. Wie is dit?</t>
+          <t>Deze filosoof, jurist en schrijver schreef 'De maakbare man', een essay over zijn eigen transitie, en romans als 'De literaire kring'. Wie kreeg de P.C. Hooft-prijs van 2020, voor beschouwend proza?</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -5770,7 +5770,7 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>De P.C. Hooft-prijs van 2021, voor poëzie, ging naar een dichter die lang in Zuid-Afrika woonde. Wie is dit?</t>
+          <t>Deze dichter woonde lang in Zuid-Afrika en werkte daar aan een universiteit. Zijn gedichten spelen met taal en identiteit. Wie kreeg de P.C. Hooft-prijs van 2021, voor poëzie?</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -5802,7 +5802,7 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>De P.C. Hooft-prijs van 2022, voor verhalend proza, ging naar een romancier van o.a. Blauwe maandagen en Tirza. Wie is dit?</t>
+          <t>Deze romancier debuteerde met 'Blauwe maandagen' en schreef 'Tirza', over een vader en zijn dochter. Hij schreef ook onder het pseudoniem Marek van der Jagt. Wie kreeg de P.C. Hooft-prijs van 2022, voor verhalend proza?</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
@@ -5834,7 +5834,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>De P.C. Hooft-prijs van 2023, voor beschouwend proza, ging naar een schrijver en evolutiebioloog van Darwins dromen. Wie is dit?</t>
+          <t>Deze schrijver en evolutiebioloog schreef 'Darwins dromen', over zijn onderzoek naar cichliden (vissen) in het Victoriameer. Wie kreeg de P.C. Hooft-prijs van 2023, voor beschouwend proza?</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -5866,7 +5866,7 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>De P.C. Hooft-prijs van 2024, voor poëzie, ging naar een eigenzinnige dichteres. Wie is dit?</t>
+          <t>Deze eigenzinnige, experimentele dichteres werd bekroond voor haar poëzie. Wie kreeg de P.C. Hooft-prijs van 2024, voor poëzie?</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr">
@@ -5898,7 +5898,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>De P.C. Hooft-prijs van 2025, voor verhalend proza, ging naar een meesterverteller uit Maassluis. Wie is dit?</t>
+          <t>Deze meesterverteller en bioloog uit Maassluis schreef 'Een vlucht regenwulpen', over een eenzame wetenschapper, en 'Het woeden der gehele wereld', over een jongen die getuige is van een moord in een Hollands stadje. Wie kreeg de P.C. Hooft-prijs van 2025, voor verhalend proza?</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
@@ -5930,7 +5930,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>De P.C. Hooft-prijs van 2026, voor beschouwend proza, ging naar een feministe en activiste; als eerste vrouw winnaar in deze categorie. Wie is dit?</t>
+          <t>Deze feministe en activiste schreef 'De schaamte voorbij' (1976), een openhartig verslag van haar leven dat een klassieker van de vrouwenbeweging werd. Ze is de eerste vrouw die de prijs voor beschouwend proza krijgt. Wie kreeg de P.C. Hooft-prijs van 2026, voor beschouwend proza?</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Nieuwe lijst: Literatuur uit de uitzendingen (31 kaarten uit de basisdataset)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GWDzH9CBKYVCbFWmsbqcR
</commit_message>
<xml_diff>
--- a/stamlijsten.xlsx
+++ b/stamlijsten.xlsx
@@ -20,7 +20,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Afgetreden bewindspersonen" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Songfestival" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literatuurprijzen" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzoektips" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literatuur uit de uitzendingen" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzoektips" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -256,6 +257,23 @@
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T11" displayName="T11" ref="A1:H65" headerRowCount="1">
   <autoFilter ref="A1:H65"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Prio"/>
+    <tableColumn id="2" name="Vraag"/>
+    <tableColumn id="3" name="Voorleesvraag"/>
+    <tableColumn id="4" name="Antwoord"/>
+    <tableColumn id="5" name="Extra"/>
+    <tableColumn id="6" name="Afbeelding"/>
+    <tableColumn id="7" name="Wiki"/>
+    <tableColumn id="8" name="Al gevraagd"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T12" displayName="T12" ref="A1:H32" headerRowCount="1">
+  <autoFilter ref="A1:H32"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Prio"/>
     <tableColumn id="2" name="Vraag"/>
@@ -7325,6 +7343,1071 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Prio</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Vraag</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Voorleesvraag</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Antwoord</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Afbeelding</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Wiki</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Al gevraagd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Roman van E.M. Forster (1924), Britse kolonie in Azië</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Deze roman van E.M. Forster uit 1924 speelt in Brits-Indië en draait om een beschuldiging na een uitstapje naar de Marabar-grotten. David Lean verfilmde hem in 1984. Hoe heet de roman?</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>A Passage to India</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr"/>
+      <c r="F2" s="9" t="inlineStr"/>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>!Marabar caves India</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Schrijfster van 'Het Hoge Nest' (Opzij Literatuurprijs 2019)</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Deze schrijfster won met 'Het Hoge Nest', over de Joodse zussen Brilleslijper die in een villa in het Gooi onderduikers verborgen, de Opzij Literatuurprijs 2019. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Roxane van Iperen</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="9" t="inlineStr"/>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>!villa forest Naarden</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Schrijfster van 'Lieve Céline', slachtoffer van een manuscriptendief</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse schrijfster werd zelf benaderd door een beruchte manuscriptendief die zich voordeed als uitgever, en probeerde hem te ontmaskeren. Ze schreef onder meer 'Lieve Céline'. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Hanna Bervoets</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="9" t="inlineStr"/>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>!manuscript typewriter</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Thrillerschrijver van 'De Hollander' (Wadden, inspecteur Cupido)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Deze thrillerschrijver laat zijn verhalen afspelen op en rond de Waddenzee, met inspecteur Cupido. Een van zijn boeken is 'De Hollander'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Matthijs Deen</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="9" t="inlineStr"/>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>!Wadden Sea mudflats</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Nijmeegse auteur en columnist van De Gelderlander</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nijmeegse auteur schrijft columns voor De Gelderlander en romans als 'Als de winter voorbij is'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Thomas Verbogt</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>!Nijmegen Waal bridge</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Schrijver van 'Gewassen vlees' en 'Publieke werken'</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Deze schrijver won tweemaal de Libris Literatuur Prijs, met 'Gewassen vlees' en 'Publieke werken', over een vioolmaker en een apotheker in het Amsterdam van de negentiende eeuw. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Thomas Rosenboom</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>!Amsterdam 19th century</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Fictieve wereld van C.S. Lewis (7 delen, kledingkast, leeuw Aslan)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>In deze zevendelige boekenreeks van C.S. Lewis stappen kinderen via een kledingkast een fictieve wereld binnen, waar de leeuw Aslan regeert. Hoe heet die wereld?</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Narnia</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr"/>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>!wardrobe snow forest lamppost</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Booker Prize 2023, 'Prophet Song'</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Deze Ierse schrijver won de Booker Prize 2023 met 'Prophet Song', een dystopische roman over een Ierland dat afglijdt naar dictatuur en burgeroorlog. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Paul Lynch</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr"/>
+      <c r="F9" s="9" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>!Dublin rain street</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>International Booker Prize 2024, 'Kairos'</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Deze Duitse schrijfster won de International Booker Prize 2024 met 'Kairos', over een verhouding tussen een jonge vrouw en een oudere man in de laatste jaren van de DDR. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Jenny Erpenbeck</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>!East Berlin 1980s</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Amerikaanse thrillerschrijver van 'Tell No One' en 'The Stranger'</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Deze Amerikaanse thrillerschrijver verkocht meer dan 80 miljoen boeken, waaronder 'Tell No One' en 'The Stranger', die door Netflix werd verfilmd. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Harlan Coben</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr"/>
+      <c r="F11" s="9" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>!New Jersey suburb night</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Amerikaanse thrillerschrijver van 'The Firm' (300 mln boeken)</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Deze Amerikaanse thrillerschrijver en oud-advocaat verkocht zo'n 300 miljoen boeken, waaronder 'The Firm' en 'The Pelican Brief'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>John Grisham</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr"/>
+      <c r="F12" s="9" t="inlineStr"/>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>!courtroom gavel</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Dystopisch subgenre van sciencefiction (Neuromancer, William Gibson)</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet het dystopische subgenre van de sciencefiction met hackers, megabedrijven en hightech in een vervallen wereld, bekend van 'Neuromancer' van William Gibson?</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Cyberpunk</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr"/>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>!neon city night rain</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Dickens: weesjongen, Fagin, zakkenrollers</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Deze roman van Charles Dickens gaat over een weesjongen die in Londen in een bende zakkenrollers van de sluwe Fagin belandt. Het boek inspireerde ook het Deventer Dickens Festijn. Hoe heet de roman?</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Oliver Twist</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr"/>
+      <c r="F14" s="9" t="inlineStr"/>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>!Victorian London street</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Dickens-roman 1839: kostschool in Yorkshire</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Deze roman van Charles Dickens uit 1839 hekelt de mishandeling van kinderen op een kostschool in Yorkshire. Hoe heet de roman, genoemd naar de hoofdpersoon?</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Nicholas Nickleby</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="9" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>!Yorkshire school 19th century</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Nederlandse auteur van 'Vloed' (hekserij)</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse schrijfster schreef 'Vloed', over hekserij en heksenvervolging, en een roman over danseres Isadora Duncan. Ze woont in Noordwijk. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Susan Smit</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr"/>
+      <c r="F16" s="9" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>!witch trial old engraving</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Nederlandse schrijfster van 'De eetclub' en 'Debet'</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse thrillerschrijfster schreef bestsellers als 'De eetclub', 'Debet' en 'De nazaten'. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Saskia Noort</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr"/>
+      <c r="F17" s="9" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>!dinner party table</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Engelse dichter ('A thing of beauty'), stierf op 25-jarige leeftijd</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Deze Engelse romantische dichter schreef 'A thing of beauty is a joy for ever', was verliefd op Fanny Brawne en stierf op 25-jarige leeftijd aan tuberculose in Rome. Wie was hij?</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>John Keats</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr"/>
+      <c r="F18" s="9" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>!Spanish Steps Rome</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Engelse dichter ('To a Skylark'), verdronk in 1822</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Deze Engelse romantische dichter schreef 'To a Skylark' en verdronk in 1822 in Italië. Zijn hart zou bij de crematie gered en bewaard zijn. Hij was getrouwd met de schrijfster van 'Frankenstein'. Wie was hij?</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Percy Bysshe Shelley</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr"/>
+      <c r="F19" s="9" t="inlineStr"/>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>!skylark bird</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Duitse schrijver van 'Die Blechtrommel' (Nobelprijs 1999)</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Deze Duitse schrijver van 'Die Blechtrommel', over een jongen die besluit niet meer te groeien, kreeg in 1999 de Nobelprijs. Later onthulde hij dat hij als tiener in de Waffen-SS had gediend. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Günter Grass</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr"/>
+      <c r="F20" s="9" t="inlineStr"/>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>!tin drum toy</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Portugese schrijver van 'De stad der blinden' (Nobelprijs 1998)</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Deze Portugese schrijver kreeg in 1998 de Nobelprijs. In zijn bekendste roman worden alle inwoners van een stad plotseling blind. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>José Saramago</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr"/>
+      <c r="F21" s="9" t="inlineStr"/>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>!Lisbon tram</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Roald Dahl: kleine fabrieksarbeiders in de chocoladefabriek</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>In 'Sjakie en de chocoladefabriek' van Roald Dahl werken in de fabriek van Willy Wonka kleine wezentjes die voor cacaobonen werken en zingende liedjes hebben. Hoe heten ze?</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Oempa Loempa's</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr"/>
+      <c r="F22" s="9" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>!chocolate factory</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Winnie de Poeh: de sombere ezel</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de sombere, pessimistische ezel uit de verhalen over Winnie de Poeh, wiens staart steeds losraakt?</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Iejoor</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Engels: Eeyore</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>!donkey grey</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Dichter van de Vijftigers ('Het leven is verrukkelijk')</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Deze dichter van de Vijftigers schreef 'Het leven is verrukkelijk' en won de P.C. Hooft-prijs. Hij overleed in 2022. Wie was hij?</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Remco Campert</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr"/>
+      <c r="F24" s="9" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>!Amsterdam café 1950s</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Schrijver van 'De Avonden', een van de Grote Drie</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Deze schrijver, een van de Grote Drie van de Nederlandse literatuur, debuteerde met 'De Avonden' en schreef 'Nader tot U'. Hij stond bekend als provocateur. Wie was hij?</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Gerard Reve</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr"/>
+      <c r="F25" s="9" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>!Amsterdam winter evening</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Schrijver van 'Philip en de anderen', 'Rituelen' en 'Allerzielen'</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Deze schrijver en reiziger schreef 'Philip en de anderen', 'Rituelen' en 'Allerzielen'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Cees Nooteboom</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr"/>
+      <c r="F26" s="9" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>!Menorca coast</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Schrijver van 'Grip' en 'Pastoralen'</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse schrijver, met een gereformeerde achtergrond, schreef 'Grip' en 'Pastoralen'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Stephan Enter</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr"/>
+      <c r="F27" s="9" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>!Dutch countryside church</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Shakespeare: tragedie over een Moorse bevelhebber</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>In deze tragedie van Shakespeare wordt een Moorse bevelhebber door de sluwe Iago zo jaloers gemaakt dat hij zijn vrouw Desdemona vermoordt. Hoe heet het stuk?</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Othello</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr"/>
+      <c r="F28" s="9" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>!Venice canal</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Shakespeare: Deense prins en de geest van zijn vader</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>In deze tragedie van Shakespeare wil een Deense prins wraak nemen op zijn oom Claudius, nadat de geest van zijn vader hem vertelt dat hij vermoord is. Hoe heet het stuk?</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Hamlet</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr"/>
+      <c r="F29" s="9" t="inlineStr"/>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>!Kronborg castle</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Thrillerschrijver van 'De macht van meneer Miller' (Gouden Strop)</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse thrillerschrijver won de Gouden Strop, onder meer met 'De macht van meneer Miller'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Charles den Tex</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr"/>
+      <c r="F30" s="9" t="inlineStr"/>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>!hangman noose rope</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Thrillerschrijver van 'Berta' (faction over Fortuyn, Srebrenica)</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse thrillerschrijver schrijft 'faction', fictie gebaseerd op echte gebeurtenissen zoals de moord op Fortuyn en Srebrenica. Een van zijn boeken heet 'Berta'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Thomas Ros</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr"/>
+      <c r="F31" s="9" t="inlineStr"/>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>!detective notebook</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Boekhandelsprijs 2025: titel van Lex Paleaux (jeugdinrichting, Canada)</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Lex Paleaux won de Boekhandelsprijs 2025 met een roman waarin een jeugdinrichting en een reis naar Canada een rol spelen. Hoe heet het boek?</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Liften naar de hemel</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr"/>
+      <c r="F32" s="9" t="inlineStr"/>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>!hitchhiking road Canada</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Literatuurlijsten samengevoegd tot één categorie Literatuur
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GWDzH9CBKYVCbFWmsbqcR
</commit_message>
<xml_diff>
--- a/stamlijsten.xlsx
+++ b/stamlijsten.xlsx
@@ -19,9 +19,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NL films" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Afgetreden bewindspersonen" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Songfestival" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literatuurprijzen" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literatuur uit de uitzendingen" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzoektips" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literatuur" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzoektips" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -255,25 +254,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T11" displayName="T11" ref="A1:H65" headerRowCount="1">
-  <autoFilter ref="A1:H65"/>
-  <tableColumns count="8">
-    <tableColumn id="1" name="Prio"/>
-    <tableColumn id="2" name="Vraag"/>
-    <tableColumn id="3" name="Voorleesvraag"/>
-    <tableColumn id="4" name="Antwoord"/>
-    <tableColumn id="5" name="Extra"/>
-    <tableColumn id="6" name="Afbeelding"/>
-    <tableColumn id="7" name="Wiki"/>
-    <tableColumn id="8" name="Al gevraagd"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
-</table>
-</file>
-
-<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T12" displayName="T12" ref="A1:H32" headerRowCount="1">
-  <autoFilter ref="A1:H32"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T11" displayName="T11" ref="A1:H96" headerRowCount="1">
+  <autoFilter ref="A1:H96"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Prio"/>
     <tableColumn id="2" name="Vraag"/>
@@ -5210,7 +5192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -7329,6 +7311,1002 @@
       </c>
       <c r="H65" s="6" t="inlineStr"/>
     </row>
+    <row r="66">
+      <c r="A66" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Roman van E.M. Forster (1924), Britse kolonie in Azië</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Deze roman van E.M. Forster uit 1924 speelt in Brits-Indië en draait om een beschuldiging na een uitstapje naar de Marabar-grotten. David Lean verfilmde hem in 1984. Hoe heet de roman?</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>A Passage to India</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr"/>
+      <c r="F66" s="9" t="inlineStr"/>
+      <c r="G66" s="8" t="inlineStr">
+        <is>
+          <t>!Marabar caves India</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Schrijfster van 'Het Hoge Nest' (Opzij Literatuurprijs 2019)</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Deze schrijfster won met 'Het Hoge Nest', over de Joodse zussen Brilleslijper die in een villa in het Gooi onderduikers verborgen, de Opzij Literatuurprijs 2019. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Roxane van Iperen</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr"/>
+      <c r="F67" s="9" t="inlineStr"/>
+      <c r="G67" s="8" t="inlineStr">
+        <is>
+          <t>!villa forest Naarden</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Schrijfster van 'Lieve Céline', slachtoffer van een manuscriptendief</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse schrijfster werd zelf benaderd door een beruchte manuscriptendief die zich voordeed als uitgever, en probeerde hem te ontmaskeren. Ze schreef onder meer 'Lieve Céline'. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Hanna Bervoets</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr"/>
+      <c r="F68" s="9" t="inlineStr"/>
+      <c r="G68" s="8" t="inlineStr">
+        <is>
+          <t>!manuscript typewriter</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Thrillerschrijver van 'De Hollander' (Wadden, inspecteur Cupido)</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Deze thrillerschrijver laat zijn verhalen afspelen op en rond de Waddenzee, met inspecteur Cupido. Een van zijn boeken is 'De Hollander'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Matthijs Deen</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr"/>
+      <c r="F69" s="9" t="inlineStr"/>
+      <c r="G69" s="8" t="inlineStr">
+        <is>
+          <t>!Wadden Sea mudflats</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Nijmeegse auteur en columnist van De Gelderlander</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nijmeegse auteur schrijft columns voor De Gelderlander en romans als 'Als de winter voorbij is'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Thomas Verbogt</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr"/>
+      <c r="F70" s="9" t="inlineStr"/>
+      <c r="G70" s="8" t="inlineStr">
+        <is>
+          <t>!Nijmegen Waal bridge</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Schrijver van 'Gewassen vlees' en 'Publieke werken'</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Deze schrijver won tweemaal de Libris Literatuur Prijs, met 'Gewassen vlees' en 'Publieke werken', over een vioolmaker en een apotheker in het Amsterdam van de negentiende eeuw. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Thomas Rosenboom</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr"/>
+      <c r="F71" s="9" t="inlineStr"/>
+      <c r="G71" s="8" t="inlineStr">
+        <is>
+          <t>!Amsterdam 19th century</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Fictieve wereld van C.S. Lewis (7 delen, kledingkast, leeuw Aslan)</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>In deze zevendelige boekenreeks van C.S. Lewis stappen kinderen via een kledingkast een fictieve wereld binnen, waar de leeuw Aslan regeert. Hoe heet die wereld?</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Narnia</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr"/>
+      <c r="F72" s="9" t="inlineStr"/>
+      <c r="G72" s="8" t="inlineStr">
+        <is>
+          <t>!wardrobe snow forest lamppost</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Booker Prize 2023, 'Prophet Song'</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Deze Ierse schrijver won de Booker Prize 2023 met 'Prophet Song', een dystopische roman over een Ierland dat afglijdt naar dictatuur en burgeroorlog. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>Paul Lynch</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr"/>
+      <c r="F73" s="9" t="inlineStr"/>
+      <c r="G73" s="8" t="inlineStr">
+        <is>
+          <t>!Dublin rain street</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>International Booker Prize 2024, 'Kairos'</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>Deze Duitse schrijfster won de International Booker Prize 2024 met 'Kairos', over een verhouding tussen een jonge vrouw en een oudere man in de laatste jaren van de DDR. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Jenny Erpenbeck</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr"/>
+      <c r="F74" s="9" t="inlineStr"/>
+      <c r="G74" s="8" t="inlineStr">
+        <is>
+          <t>!East Berlin 1980s</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Amerikaanse thrillerschrijver van 'Tell No One' en 'The Stranger'</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Deze Amerikaanse thrillerschrijver verkocht meer dan 80 miljoen boeken, waaronder 'Tell No One' en 'The Stranger', die door Netflix werd verfilmd. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>Harlan Coben</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr"/>
+      <c r="F75" s="9" t="inlineStr"/>
+      <c r="G75" s="8" t="inlineStr">
+        <is>
+          <t>!New Jersey suburb night</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>Amerikaanse thrillerschrijver van 'The Firm' (300 mln boeken)</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>Deze Amerikaanse thrillerschrijver en oud-advocaat verkocht zo'n 300 miljoen boeken, waaronder 'The Firm' en 'The Pelican Brief'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>John Grisham</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr"/>
+      <c r="F76" s="9" t="inlineStr"/>
+      <c r="G76" s="8" t="inlineStr">
+        <is>
+          <t>!courtroom gavel</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Dystopisch subgenre van sciencefiction (Neuromancer, William Gibson)</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet het dystopische subgenre van de sciencefiction met hackers, megabedrijven en hightech in een vervallen wereld, bekend van 'Neuromancer' van William Gibson?</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>Cyberpunk</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr"/>
+      <c r="F77" s="9" t="inlineStr"/>
+      <c r="G77" s="8" t="inlineStr">
+        <is>
+          <t>!neon city night rain</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Dickens: weesjongen, Fagin, zakkenrollers</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>Deze roman van Charles Dickens gaat over een weesjongen die in Londen in een bende zakkenrollers van de sluwe Fagin belandt. Het boek inspireerde ook het Deventer Dickens Festijn. Hoe heet de roman?</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>Oliver Twist</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr"/>
+      <c r="F78" s="9" t="inlineStr"/>
+      <c r="G78" s="8" t="inlineStr">
+        <is>
+          <t>!Victorian London street</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Dickens-roman 1839: kostschool in Yorkshire</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Deze roman van Charles Dickens uit 1839 hekelt de mishandeling van kinderen op een kostschool in Yorkshire. Hoe heet de roman, genoemd naar de hoofdpersoon?</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>Nicholas Nickleby</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr"/>
+      <c r="F79" s="9" t="inlineStr"/>
+      <c r="G79" s="8" t="inlineStr">
+        <is>
+          <t>!Yorkshire school 19th century</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>Nederlandse auteur van 'Vloed' (hekserij)</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse schrijfster schreef 'Vloed', over hekserij en heksenvervolging, en een roman over danseres Isadora Duncan. Ze woont in Noordwijk. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>Susan Smit</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr"/>
+      <c r="F80" s="9" t="inlineStr"/>
+      <c r="G80" s="8" t="inlineStr">
+        <is>
+          <t>!witch trial old engraving</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Nederlandse schrijfster van 'De eetclub' en 'Debet'</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse thrillerschrijfster schreef bestsellers als 'De eetclub', 'Debet' en 'De nazaten'. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>Saskia Noort</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr"/>
+      <c r="F81" s="9" t="inlineStr"/>
+      <c r="G81" s="8" t="inlineStr">
+        <is>
+          <t>!dinner party table</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>Engelse dichter ('A thing of beauty'), stierf op 25-jarige leeftijd</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>Deze Engelse romantische dichter schreef 'A thing of beauty is a joy for ever', was verliefd op Fanny Brawne en stierf op 25-jarige leeftijd aan tuberculose in Rome. Wie was hij?</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>John Keats</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr"/>
+      <c r="F82" s="9" t="inlineStr"/>
+      <c r="G82" s="8" t="inlineStr">
+        <is>
+          <t>!Spanish Steps Rome</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Engelse dichter ('To a Skylark'), verdronk in 1822</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Deze Engelse romantische dichter schreef 'To a Skylark' en verdronk in 1822 in Italië. Zijn hart zou bij de crematie gered en bewaard zijn. Hij was getrouwd met de schrijfster van 'Frankenstein'. Wie was hij?</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>Percy Bysshe Shelley</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr"/>
+      <c r="F83" s="9" t="inlineStr"/>
+      <c r="G83" s="8" t="inlineStr">
+        <is>
+          <t>!skylark bird</t>
+        </is>
+      </c>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>Duitse schrijver van 'Die Blechtrommel' (Nobelprijs 1999)</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>Deze Duitse schrijver van 'Die Blechtrommel', over een jongen die besluit niet meer te groeien, kreeg in 1999 de Nobelprijs. Later onthulde hij dat hij als tiener in de Waffen-SS had gediend. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Günter Grass</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr"/>
+      <c r="F84" s="9" t="inlineStr"/>
+      <c r="G84" s="8" t="inlineStr">
+        <is>
+          <t>!tin drum toy</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Portugese schrijver van 'De stad der blinden' (Nobelprijs 1998)</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>Deze Portugese schrijver kreeg in 1998 de Nobelprijs. In zijn bekendste roman worden alle inwoners van een stad plotseling blind. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>José Saramago</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr"/>
+      <c r="F85" s="9" t="inlineStr"/>
+      <c r="G85" s="8" t="inlineStr">
+        <is>
+          <t>!Lisbon tram</t>
+        </is>
+      </c>
+      <c r="H85" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Roald Dahl: kleine fabrieksarbeiders in de chocoladefabriek</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>In 'Sjakie en de chocoladefabriek' van Roald Dahl werken in de fabriek van Willy Wonka kleine wezentjes die voor cacaobonen werken en zingende liedjes hebben. Hoe heten ze?</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Oempa Loempa's</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="inlineStr"/>
+      <c r="F86" s="9" t="inlineStr"/>
+      <c r="G86" s="8" t="inlineStr">
+        <is>
+          <t>!chocolate factory</t>
+        </is>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Winnie de Poeh: de sombere ezel</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de sombere, pessimistische ezel uit de verhalen over Winnie de Poeh, wiens staart steeds losraakt?</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>Iejoor</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
+          <t>Engels: Eeyore</t>
+        </is>
+      </c>
+      <c r="F87" s="9" t="inlineStr"/>
+      <c r="G87" s="8" t="inlineStr">
+        <is>
+          <t>!donkey grey</t>
+        </is>
+      </c>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>Dichter van de Vijftigers ('Het leven is verrukkelijk')</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>Deze dichter van de Vijftigers schreef 'Het leven is verrukkelijk' en won de P.C. Hooft-prijs. Hij overleed in 2022. Wie was hij?</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Remco Campert</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="inlineStr"/>
+      <c r="F88" s="9" t="inlineStr"/>
+      <c r="G88" s="8" t="inlineStr">
+        <is>
+          <t>!Amsterdam café 1950s</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>Schrijver van 'De Avonden', een van de Grote Drie</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>Deze schrijver, een van de Grote Drie van de Nederlandse literatuur, debuteerde met 'De Avonden' en schreef 'Nader tot U'. Hij stond bekend als provocateur. Wie was hij?</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>Gerard Reve</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="inlineStr"/>
+      <c r="F89" s="9" t="inlineStr"/>
+      <c r="G89" s="8" t="inlineStr">
+        <is>
+          <t>!Amsterdam winter evening</t>
+        </is>
+      </c>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>Schrijver van 'Philip en de anderen', 'Rituelen' en 'Allerzielen'</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>Deze schrijver en reiziger schreef 'Philip en de anderen', 'Rituelen' en 'Allerzielen'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Cees Nooteboom</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr"/>
+      <c r="F90" s="9" t="inlineStr"/>
+      <c r="G90" s="8" t="inlineStr">
+        <is>
+          <t>!Menorca coast</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>Schrijver van 'Grip' en 'Pastoralen'</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse schrijver, met een gereformeerde achtergrond, schreef 'Grip' en 'Pastoralen'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>Stephan Enter</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr"/>
+      <c r="F91" s="9" t="inlineStr"/>
+      <c r="G91" s="8" t="inlineStr">
+        <is>
+          <t>!Dutch countryside church</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>Shakespeare: tragedie over een Moorse bevelhebber</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>In deze tragedie van Shakespeare wordt een Moorse bevelhebber door de sluwe Iago zo jaloers gemaakt dat hij zijn vrouw Desdemona vermoordt. Hoe heet het stuk?</t>
+        </is>
+      </c>
+      <c r="D92" s="8" t="inlineStr">
+        <is>
+          <t>Othello</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr"/>
+      <c r="F92" s="9" t="inlineStr"/>
+      <c r="G92" s="8" t="inlineStr">
+        <is>
+          <t>!Venice canal</t>
+        </is>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>Shakespeare: Deense prins en de geest van zijn vader</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>In deze tragedie van Shakespeare wil een Deense prins wraak nemen op zijn oom Claudius, nadat de geest van zijn vader hem vertelt dat hij vermoord is. Hoe heet het stuk?</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>Hamlet</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr"/>
+      <c r="F93" s="9" t="inlineStr"/>
+      <c r="G93" s="8" t="inlineStr">
+        <is>
+          <t>!Kronborg castle</t>
+        </is>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>Thrillerschrijver van 'De macht van meneer Miller' (Gouden Strop)</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse thrillerschrijver won de Gouden Strop, onder meer met 'De macht van meneer Miller'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D94" s="8" t="inlineStr">
+        <is>
+          <t>Charles den Tex</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr"/>
+      <c r="F94" s="9" t="inlineStr"/>
+      <c r="G94" s="8" t="inlineStr">
+        <is>
+          <t>!hangman noose rope</t>
+        </is>
+      </c>
+      <c r="H94" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>Thrillerschrijver van 'Berta' (faction over Fortuyn, Srebrenica)</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse thrillerschrijver schrijft 'faction', fictie gebaseerd op echte gebeurtenissen zoals de moord op Fortuyn en Srebrenica. Een van zijn boeken heet 'Berta'. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>Thomas Ros</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="inlineStr"/>
+      <c r="F95" s="9" t="inlineStr"/>
+      <c r="G95" s="8" t="inlineStr">
+        <is>
+          <t>!detective notebook</t>
+        </is>
+      </c>
+      <c r="H95" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>Boekhandelsprijs 2025: titel van Lex Paleaux (jeugdinrichting, Canada)</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>Lex Paleaux won de Boekhandelsprijs 2025 met een roman waarin een jeugdinrichting en een reis naar Canada een rol spelen. Hoe heet het boek?</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>Liften naar de hemel</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr"/>
+      <c r="F96" s="9" t="inlineStr"/>
+      <c r="G96" s="8" t="inlineStr">
+        <is>
+          <t>!hitchhiking road Canada</t>
+        </is>
+      </c>
+      <c r="H96" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -7338,1071 +8316,6 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H32"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Prio</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Vraag</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Voorleesvraag</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Antwoord</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Extra</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Afbeelding</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Wiki</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Al gevraagd</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>Roman van E.M. Forster (1924), Britse kolonie in Azië</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>Deze roman van E.M. Forster uit 1924 speelt in Brits-Indië en draait om een beschuldiging na een uitstapje naar de Marabar-grotten. David Lean verfilmde hem in 1984. Hoe heet de roman?</t>
-        </is>
-      </c>
-      <c r="D2" s="8" t="inlineStr">
-        <is>
-          <t>A Passage to India</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr"/>
-      <c r="F2" s="9" t="inlineStr"/>
-      <c r="G2" s="8" t="inlineStr">
-        <is>
-          <t>!Marabar caves India</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Schrijfster van 'Het Hoge Nest' (Opzij Literatuurprijs 2019)</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Deze schrijfster won met 'Het Hoge Nest', over de Joodse zussen Brilleslijper die in een villa in het Gooi onderduikers verborgen, de Opzij Literatuurprijs 2019. Wie is zij?</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Roxane van Iperen</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="9" t="inlineStr"/>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>!villa forest Naarden</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Schrijfster van 'Lieve Céline', slachtoffer van een manuscriptendief</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Deze Nederlandse schrijfster werd zelf benaderd door een beruchte manuscriptendief die zich voordeed als uitgever, en probeerde hem te ontmaskeren. Ze schreef onder meer 'Lieve Céline'. Wie is zij?</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Hanna Bervoets</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="9" t="inlineStr"/>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>!manuscript typewriter</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Thrillerschrijver van 'De Hollander' (Wadden, inspecteur Cupido)</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Deze thrillerschrijver laat zijn verhalen afspelen op en rond de Waddenzee, met inspecteur Cupido. Een van zijn boeken is 'De Hollander'. Wie is hij?</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Matthijs Deen</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="9" t="inlineStr"/>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>!Wadden Sea mudflats</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Nijmeegse auteur en columnist van De Gelderlander</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Deze Nijmeegse auteur schrijft columns voor De Gelderlander en romans als 'Als de winter voorbij is'. Wie is hij?</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Thomas Verbogt</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="9" t="inlineStr"/>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>!Nijmegen Waal bridge</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Schrijver van 'Gewassen vlees' en 'Publieke werken'</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Deze schrijver won tweemaal de Libris Literatuur Prijs, met 'Gewassen vlees' en 'Publieke werken', over een vioolmaker en een apotheker in het Amsterdam van de negentiende eeuw. Wie is hij?</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>Thomas Rosenboom</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="9" t="inlineStr"/>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>!Amsterdam 19th century</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Fictieve wereld van C.S. Lewis (7 delen, kledingkast, leeuw Aslan)</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>In deze zevendelige boekenreeks van C.S. Lewis stappen kinderen via een kledingkast een fictieve wereld binnen, waar de leeuw Aslan regeert. Hoe heet die wereld?</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Narnia</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="9" t="inlineStr"/>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>!wardrobe snow forest lamppost</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Booker Prize 2023, 'Prophet Song'</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Deze Ierse schrijver won de Booker Prize 2023 met 'Prophet Song', een dystopische roman over een Ierland dat afglijdt naar dictatuur en burgeroorlog. Wie is hij?</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Paul Lynch</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="9" t="inlineStr"/>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>!Dublin rain street</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>International Booker Prize 2024, 'Kairos'</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Deze Duitse schrijfster won de International Booker Prize 2024 met 'Kairos', over een verhouding tussen een jonge vrouw en een oudere man in de laatste jaren van de DDR. Wie is zij?</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Jenny Erpenbeck</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="9" t="inlineStr"/>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>!East Berlin 1980s</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Amerikaanse thrillerschrijver van 'Tell No One' en 'The Stranger'</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Deze Amerikaanse thrillerschrijver verkocht meer dan 80 miljoen boeken, waaronder 'Tell No One' en 'The Stranger', die door Netflix werd verfilmd. Wie is hij?</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Harlan Coben</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="9" t="inlineStr"/>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>!New Jersey suburb night</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Amerikaanse thrillerschrijver van 'The Firm' (300 mln boeken)</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Deze Amerikaanse thrillerschrijver en oud-advocaat verkocht zo'n 300 miljoen boeken, waaronder 'The Firm' en 'The Pelican Brief'. Wie is hij?</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>John Grisham</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="9" t="inlineStr"/>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>!courtroom gavel</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Dystopisch subgenre van sciencefiction (Neuromancer, William Gibson)</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Hoe heet het dystopische subgenre van de sciencefiction met hackers, megabedrijven en hightech in een vervallen wereld, bekend van 'Neuromancer' van William Gibson?</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Cyberpunk</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="9" t="inlineStr"/>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>!neon city night rain</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Dickens: weesjongen, Fagin, zakkenrollers</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Deze roman van Charles Dickens gaat over een weesjongen die in Londen in een bende zakkenrollers van de sluwe Fagin belandt. Het boek inspireerde ook het Deventer Dickens Festijn. Hoe heet de roman?</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Oliver Twist</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr"/>
-      <c r="F14" s="9" t="inlineStr"/>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>!Victorian London street</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>Dickens-roman 1839: kostschool in Yorkshire</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>Deze roman van Charles Dickens uit 1839 hekelt de mishandeling van kinderen op een kostschool in Yorkshire. Hoe heet de roman, genoemd naar de hoofdpersoon?</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Nicholas Nickleby</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="9" t="inlineStr"/>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>!Yorkshire school 19th century</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Nederlandse auteur van 'Vloed' (hekserij)</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>Deze Nederlandse schrijfster schreef 'Vloed', over hekserij en heksenvervolging, en een roman over danseres Isadora Duncan. Ze woont in Noordwijk. Wie is zij?</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Susan Smit</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="9" t="inlineStr"/>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>!witch trial old engraving</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Nederlandse schrijfster van 'De eetclub' en 'Debet'</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>Deze Nederlandse thrillerschrijfster schreef bestsellers als 'De eetclub', 'Debet' en 'De nazaten'. Wie is zij?</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Saskia Noort</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr"/>
-      <c r="F17" s="9" t="inlineStr"/>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>!dinner party table</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Engelse dichter ('A thing of beauty'), stierf op 25-jarige leeftijd</t>
-        </is>
-      </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Deze Engelse romantische dichter schreef 'A thing of beauty is a joy for ever', was verliefd op Fanny Brawne en stierf op 25-jarige leeftijd aan tuberculose in Rome. Wie was hij?</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>John Keats</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr"/>
-      <c r="F18" s="9" t="inlineStr"/>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>!Spanish Steps Rome</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>Engelse dichter ('To a Skylark'), verdronk in 1822</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>Deze Engelse romantische dichter schreef 'To a Skylark' en verdronk in 1822 in Italië. Zijn hart zou bij de crematie gered en bewaard zijn. Hij was getrouwd met de schrijfster van 'Frankenstein'. Wie was hij?</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>Percy Bysshe Shelley</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr"/>
-      <c r="F19" s="9" t="inlineStr"/>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>!skylark bird</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>Duitse schrijver van 'Die Blechtrommel' (Nobelprijs 1999)</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Deze Duitse schrijver van 'Die Blechtrommel', over een jongen die besluit niet meer te groeien, kreeg in 1999 de Nobelprijs. Later onthulde hij dat hij als tiener in de Waffen-SS had gediend. Wie is hij?</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>Günter Grass</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr"/>
-      <c r="F20" s="9" t="inlineStr"/>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>!tin drum toy</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>Portugese schrijver van 'De stad der blinden' (Nobelprijs 1998)</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>Deze Portugese schrijver kreeg in 1998 de Nobelprijs. In zijn bekendste roman worden alle inwoners van een stad plotseling blind. Wie is hij?</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>José Saramago</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr"/>
-      <c r="F21" s="9" t="inlineStr"/>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>!Lisbon tram</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Roald Dahl: kleine fabrieksarbeiders in de chocoladefabriek</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>In 'Sjakie en de chocoladefabriek' van Roald Dahl werken in de fabriek van Willy Wonka kleine wezentjes die voor cacaobonen werken en zingende liedjes hebben. Hoe heten ze?</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>Oempa Loempa's</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="inlineStr"/>
-      <c r="F22" s="9" t="inlineStr"/>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>!chocolate factory</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Winnie de Poeh: de sombere ezel</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>Hoe heet de sombere, pessimistische ezel uit de verhalen over Winnie de Poeh, wiens staart steeds losraakt?</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>Iejoor</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Engels: Eeyore</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr"/>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>!donkey grey</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
-        <is>
-          <t>Dichter van de Vijftigers ('Het leven is verrukkelijk')</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>Deze dichter van de Vijftigers schreef 'Het leven is verrukkelijk' en won de P.C. Hooft-prijs. Hij overleed in 2022. Wie was hij?</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>Remco Campert</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr"/>
-      <c r="F24" s="9" t="inlineStr"/>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>!Amsterdam café 1950s</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>Schrijver van 'De Avonden', een van de Grote Drie</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Deze schrijver, een van de Grote Drie van de Nederlandse literatuur, debuteerde met 'De Avonden' en schreef 'Nader tot U'. Hij stond bekend als provocateur. Wie was hij?</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>Gerard Reve</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr"/>
-      <c r="F25" s="9" t="inlineStr"/>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>!Amsterdam winter evening</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>Schrijver van 'Philip en de anderen', 'Rituelen' en 'Allerzielen'</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>Deze schrijver en reiziger schreef 'Philip en de anderen', 'Rituelen' en 'Allerzielen'. Wie is hij?</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>Cees Nooteboom</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr"/>
-      <c r="F26" s="9" t="inlineStr"/>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>!Menorca coast</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Schrijver van 'Grip' en 'Pastoralen'</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Deze Nederlandse schrijver, met een gereformeerde achtergrond, schreef 'Grip' en 'Pastoralen'. Wie is hij?</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>Stephan Enter</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr"/>
-      <c r="F27" s="9" t="inlineStr"/>
-      <c r="G27" s="8" t="inlineStr">
-        <is>
-          <t>!Dutch countryside church</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>Shakespeare: tragedie over een Moorse bevelhebber</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>In deze tragedie van Shakespeare wordt een Moorse bevelhebber door de sluwe Iago zo jaloers gemaakt dat hij zijn vrouw Desdemona vermoordt. Hoe heet het stuk?</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>Othello</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr"/>
-      <c r="F28" s="9" t="inlineStr"/>
-      <c r="G28" s="8" t="inlineStr">
-        <is>
-          <t>!Venice canal</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>Shakespeare: Deense prins en de geest van zijn vader</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>In deze tragedie van Shakespeare wil een Deense prins wraak nemen op zijn oom Claudius, nadat de geest van zijn vader hem vertelt dat hij vermoord is. Hoe heet het stuk?</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>Hamlet</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr"/>
-      <c r="F29" s="9" t="inlineStr"/>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>!Kronborg castle</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Thrillerschrijver van 'De macht van meneer Miller' (Gouden Strop)</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Deze Nederlandse thrillerschrijver won de Gouden Strop, onder meer met 'De macht van meneer Miller'. Wie is hij?</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Charles den Tex</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr"/>
-      <c r="F30" s="9" t="inlineStr"/>
-      <c r="G30" s="8" t="inlineStr">
-        <is>
-          <t>!hangman noose rope</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>Thrillerschrijver van 'Berta' (faction over Fortuyn, Srebrenica)</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>Deze Nederlandse thrillerschrijver schrijft 'faction', fictie gebaseerd op echte gebeurtenissen zoals de moord op Fortuyn en Srebrenica. Een van zijn boeken heet 'Berta'. Wie is hij?</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>Thomas Ros</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr"/>
-      <c r="F31" s="9" t="inlineStr"/>
-      <c r="G31" s="8" t="inlineStr">
-        <is>
-          <t>!detective notebook</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>Boekhandelsprijs 2025: titel van Lex Paleaux (jeugdinrichting, Canada)</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Lex Paleaux won de Boekhandelsprijs 2025 met een roman waarin een jeugdinrichting en een reis naar Canada een rol spelen. Hoe heet het boek?</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>Liften naar de hemel</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr"/>
-      <c r="F32" s="9" t="inlineStr"/>
-      <c r="G32" s="8" t="inlineStr">
-        <is>
-          <t>!hitchhiking road Canada</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Nieuwe lijst: Sport (gericht op vraagtypes die fout gingen of opgezocht moesten worden)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GWDzH9CBKYVCbFWmsbqcR
</commit_message>
<xml_diff>
--- a/stamlijsten.xlsx
+++ b/stamlijsten.xlsx
@@ -20,7 +20,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Afgetreden bewindspersonen" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Songfestival" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literatuur" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzoektips" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sport" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opzoektips" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -256,6 +257,23 @@
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T11" displayName="T11" ref="A1:H96" headerRowCount="1">
   <autoFilter ref="A1:H96"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Prio"/>
+    <tableColumn id="2" name="Vraag"/>
+    <tableColumn id="3" name="Voorleesvraag"/>
+    <tableColumn id="4" name="Antwoord"/>
+    <tableColumn id="5" name="Extra"/>
+    <tableColumn id="6" name="Afbeelding"/>
+    <tableColumn id="7" name="Wiki"/>
+    <tableColumn id="8" name="Al gevraagd"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T12" displayName="T12" ref="A1:H99" headerRowCount="1">
+  <autoFilter ref="A1:H99"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Prio"/>
     <tableColumn id="2" name="Vraag"/>
@@ -8321,6 +8339,3011 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H99"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Prio</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Vraag</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Voorleesvraag</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Antwoord</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Afbeelding</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Wiki</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Al gevraagd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Rugby: spelhervatting waarbij twee groepen tegen elkaar in duwen</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>In het rugby wordt het spel na een kleine overtreding hervat doordat de voorwaartsen van beide teams gebukt in elkaar grijpen en tegen elkaar in duwen, terwijl de bal ertussen wordt ingegooid. Hoe heet dit?</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Scrum</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Niet: huddle (overleg bij American football)</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr"/>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>?scrum rugby</t>
+        </is>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Rugby: inworp vanaf de zijlijn, spelers worden opgetild</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>In het rugby gooit een speler de bal na een uitbal vanaf de zijlijn in tussen twee rijen spelers, die elkaar optillen om hem te vangen. Hoe heet dit?</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Line-out</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="9" t="inlineStr"/>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>?line-out rugby</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Rugby: Maori-dans van de All Blacks voor de wedstrijd</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Het Nieuw-Zeelandse rugbyteam, de All Blacks, voert voor elke wedstrijd een traditionele Maori-strijddans op met stampen, schreeuwen en uitgestoken tongen. Hoe heet die dans?</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Haka</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="9" t="inlineStr"/>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Haka</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Rugby: bal achter de doellijn op de grond drukken (5 punten)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>In het rugby scoor je de meeste punten door de bal achter de doellijn van de tegenstander op de grond te drukken. Hoe heet zo'n score?</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Try</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Te vergelijken met een touchdown</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr"/>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>?try rugby score</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>American football: kort overleg in een kring voor elke spelpoging</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>In het American football gaan de spelers voor elke spelpoging even in een kring staan om de volgende tactiek af te spreken. Hoe heet dat?</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Huddle</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Niet verwarren met de scrum bij rugby</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>?huddle American football</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Tennis: beslissende game bij 6-6</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>In het tennis wordt een set bij een stand van 6-6 meestal beslist met een speciale game met afwijkende telling, waarin je tot minstens zeven punten speelt. Hoe heet die game?</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Tiebreak</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>Niet: matchpoint</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>?tiebreak tennis</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Tennis: 40-40, Franse oorsprong</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het tennis de stand 40-40, waarna een speler twee punten op rij moet winnen? Het woord komt via het Engels van het Franse 'à deux'.</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Deuce</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr"/>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>?deuce tennis</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Tennis: voorwaartse draai op de bal (Magnus-effect)</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het tennis de voorwaartse draai die je de bal meegeeft, waardoor hij door het Magnus-effect sneller daalt en hoog opspringt?</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Topspin</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Niet alleen 'spin'. Tegenovergestelde: slice/backspin</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>?topspin tennis</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Tennis: bal met achterwaartse draai, laag stuitend</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het tennis een slag waarbij je de bal van boven naar onder raakt, zodat hij achterwaarts draait en laag blijft na het stuiten?</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Slice</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr"/>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>?slice tennis backhand</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Tennis: opslag die de ontvanger niet raakt</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het tennis een opslag die zo goed is dat de ontvanger de bal niet eens kan raken?</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Ace</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr"/>
+      <c r="F11" s="9" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>?ace tennis serve</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Tennis: opslag die het net raakt en goed is, wordt overgespeeld</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>In het tennis raakt een opslag het net maar valt hij wel in het juiste vak. Hij wordt dan overgedaan. Welk Engels woord roept de scheidsrechter?</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Let</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr"/>
+      <c r="F12" s="9" t="inlineStr"/>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>?let tennis net</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Tennis: hoge bal over de tegenstander aan het net</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het tennis een hoge boogbal over een tegenstander die aan het net staat?</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Lob</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr"/>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>?lob tennis</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Tennis: game winnen op de opslag van de tegenstander</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet het in het tennis als je een game wint terwijl je tegenstander serveert?</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Break</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr"/>
+      <c r="F14" s="9" t="inlineStr"/>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>?break point tennis</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Racketsport uit 1965 met paddle, plastic bal en 'kitchen'</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Deze racketsport ontstond in 1965 in de Verenigde Staten. Je speelt met een houten of composiet paddle en een plastic bal met gaatjes, op een klein veld met een zone bij het net die de 'kitchen' heet, tot elf punten. Hoe heet de sport?</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Pickleball</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Niet: padel (met glazen wanden)</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr"/>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Pickleball</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Racketsport met glazen wanden, populair in Spanje</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Deze racketsport, een mengvorm van tennis en squash, wordt in dubbels gespeeld op een kleine baan met glazen wanden die je mag gebruiken. Ze is enorm populair in Spanje en Argentinië. Hoe heet hij?</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>Padel</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Niet: pickleball</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr"/>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>Padel</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Badminton: het 'balletje' met veren</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet het projectiel waarmee badminton wordt gespeeld, met een kurken dop en zestien ganzenveren?</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Shuttle</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr"/>
+      <c r="F17" s="9" t="inlineStr"/>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>?shuttlecock badminton</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Drafsport: persoon die het paard ment</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>In de drafsport zit iemand in een licht karretje achter het paard en ment het. Hoe heet die persoon? Het woord komt uit het Frans.</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Pikeur</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Niet: jockey (die rijdt bij galop op het paard)</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr"/>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>!harness racing</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Drafsport: het lichte karretje</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet het lichte tweewielige karretje dat in de drafsport door het paard wordt voortgetrokken?</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Sulky</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr"/>
+      <c r="F19" s="9" t="inlineStr"/>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>!harness racing</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Paardensport: dressuur, springen en cross-country (vroeger 'military')</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Deze paardensport combineert dressuur, springen en een cross-country door het terrein. Vroeger heette ze 'military'. Wat is de Engelse naam?</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Eventing</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr"/>
+      <c r="F20" s="9" t="inlineStr"/>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>!cross country horse jump</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Paardensport: acrobatiek op een galopperend paard</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Bij deze sport doen sporters turnoefeningen op de rug van een paard dat aan een longe in een cirkel galoppeert. Hoe heet de sport?</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Voltige</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr"/>
+      <c r="F21" s="9" t="inlineStr"/>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>!equestrian vaulting</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Paardenrace in Epsom sinds 1780, naar een graaf</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Deze beroemde paardenrace in Epsom bestaat sinds 1780 en is genoemd naar een Engelse graaf. Het woord wordt nu ook gebruikt voor een wedstrijd tussen stadsgenoten. Hoe heet hij?</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Derby</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr"/>
+      <c r="F22" s="9" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>!Epsom Downs racecourse</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Hindernisrace (paarden of atletiek) met water</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet een wedloop met hindernissen en een waterbak, bij de atletiek over drieduizend meter, oorspronkelijk een paardenrace van kerktoren naar kerktoren?</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Steeplechase</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr"/>
+      <c r="F23" s="9" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>?steeplechase athletics water jump</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Judo: band om de jas, geeft niveau aan</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet bij judo en karate de band om de jas, waarvan de kleur het niveau aangeeft?</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Obi</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr"/>
+      <c r="F24" s="9" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>?obi judo belt</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Judo: de mat</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de Japanse mat waarop judo wordt beoefend, vroeger van rijststro en nu van schuim met vinyl?</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Tatami</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr"/>
+      <c r="F25" s="9" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>?tatami judo</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Judo: de witte of blauwe jas</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet het pak waarin judoka's vechten, met een dikke katoenen jas?</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Judogi</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr"/>
+      <c r="F26" s="9" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>Judogi</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Judo: volle score, beslist de partij</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet bij judo de hoogste score, waarmee de partij meteen is beslist?</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Ippon</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr"/>
+      <c r="F27" s="9" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>?ippon judo</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Vechtsport: oefenruimte</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de oefenruimte van een Japanse vechtsport als judo of karate?</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Dojo</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr"/>
+      <c r="F28" s="9" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Dojo</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Japanse vechtkunst van Morihei Ueshiba (ontwijken, klemmen)</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Deze Japanse verdedigingskunst werd ontwikkeld door Morihei Ueshiba. Je gebruikt de kracht van de aanvaller tegen hem met ontwijkingen, worpen en klemtechnieken. Hoe heet hij?</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Aikido</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr"/>
+      <c r="F29" s="9" t="inlineStr"/>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Aikido</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Japanse vechtkunst van de samurai, basis voor judo</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Uit deze Japanse vechtkunst van de samurai, met worpen, klemmen en slagen, ontwikkelde Jigoro Kano later het judo. Hoe heet hij?</t>
+        </is>
+      </c>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>Jiu-jitsu</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr"/>
+      <c r="F30" s="9" t="inlineStr"/>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>Jiu-jitsu</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Oprichter van het judo (1882)</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Deze Japanner richtte in 1882 het judo op, de 'zachte weg', als sport afgeleid van jiu-jitsu. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Jigoro Kano</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr"/>
+      <c r="F31" s="9" t="inlineStr"/>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Kanō Jigorō</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Nederlandse judoka, olympisch goud Tokio 1964</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Deze Utrechtse judoka versloeg in 1964 in Tokio de Japanner Kaminaga in de open klasse en won olympisch goud. Een schok voor Japan. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>Anton Geesink</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr"/>
+      <c r="F32" s="9" t="inlineStr"/>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Anton Geesink</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Sumo: hoogste rang</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de hoogste rang in het Japanse sumoworstelen?</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Yokozuna</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr"/>
+      <c r="F33" s="9" t="inlineStr"/>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Yokozuna</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Koreaanse vechtsport met veel trappen (olympisch)</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Deze olympische vechtsport uit Korea staat bekend om hoge trappen en sprongtrappen. Hoe heet hij?</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>Taekwondo</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr"/>
+      <c r="F34" s="9" t="inlineStr"/>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Taekwondo</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Japanse zwaardvechtkunst met bamboe zwaarden</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Bij deze Japanse vechtkunst vechten sporters met harnas en masker met bamboe zwaarden, shinai genoemd. Hoe heet hij?</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Kendo</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr"/>
+      <c r="F35" s="9" t="inlineStr"/>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Kendo</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Wielrennen: schuin achter elkaar rijden bij zijwind</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het wielrennen de schuine rij renners die bij zijwind ontstaat, waarbij iedereen beschutting zoekt achter een ander?</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>Waaier</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr"/>
+      <c r="F36" s="9" t="inlineStr"/>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>!crosswind cycling peloton</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Wielrennen: plotselinge versnelling (Frans)</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het wielrennen een plotselinge versnelling om een gat te slaan, met een Franse term?</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Démarrage</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr"/>
+      <c r="F37" s="9" t="inlineStr"/>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>!cycling attack climb</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Wielrennen: verzorger van de renners</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het wielrennen de verzorger die renners masseert en bidons en eten aangeeft? Het woord komt uit het Frans.</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>Soigneur</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr"/>
+      <c r="F38" s="9" t="inlineStr"/>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>!cycling team car feeding</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Wielrennen: knecht die werkt voor de kopman</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het wielrennen een knecht die zichzelf opoffert voor de kopman, met een Franse term die 'huisbediende' betekent?</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Domestique</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr"/>
+      <c r="F39" s="9" t="inlineStr"/>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>!cycling peloton</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>Wielrennen: laatste in het algemeen klassement van de Tour</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de renner die als allerlaatste in het algemeen klassement van de Tour de France eindigt, vertaald de 'rode lantaarn'?</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Lanterne rouge</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr"/>
+      <c r="F40" s="9" t="inlineStr"/>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>!red lantern</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Wielrennen: drinkbus</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de drinkbus aan de fiets van een wielrenner?</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Bidon</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr"/>
+      <c r="F41" s="9" t="inlineStr"/>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>!cycling water bottle</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>Baanwielrennen: sprint achter een gangmaker op een motortje (Japans)</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Bij dit Japanse baanwielrennummer rijden de renners eerst achter een gangmaker op een gemotoriseerde fiets, waarna ze de laatste ronden sprinten. Harrie Lavreysen won hierin olympisch goud. Hoe heet het?</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Keirin</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr"/>
+      <c r="F42" s="9" t="inlineStr"/>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>?keirin track cycling</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Gemotoriseerde gangmakersfiets bij de baan</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de gemotoriseerde fiets waarachter baanwielrenners en stayers rijden?</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Derny</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr"/>
+      <c r="F43" s="9" t="inlineStr"/>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>Derny</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>Schaken: koning en toren tegelijk verplaatsen</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de schaakzet waarbij koning en toren tegelijk worden verplaatst?</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Rokade</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr"/>
+      <c r="F44" s="9" t="inlineStr"/>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>?castling chess</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Schaken: pion slaat pion die twee velden sprong</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de speciale schaakregel waarbij een pion een andere pion slaat die net twee velden vooruit is gegaan, alsof die er maar één had gezet? Het is Frans voor 'in het voorbijgaan'.</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>En passant</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr"/>
+      <c r="F45" s="9" t="inlineStr"/>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>?en passant chess</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>Schaken: opening waarin je een pion offert</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet een schaakopening waarin je bewust een pion offert voor een betere positie?</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>Gambiet</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="inlineStr"/>
+      <c r="F46" s="9" t="inlineStr"/>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>?gambit chess opening</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Schaken: elke zet verslechtert je stelling (Duits)</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het schaken de situatie waarin je verplicht bent een zet te doen, terwijl elke zet je stelling verslechtert? Het is een Duits woord.</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Zugzwang</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr"/>
+      <c r="F47" s="9" t="inlineStr"/>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>?zugzwang chess</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Schaken: niet schaak staan maar geen zet meer kunnen doen</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het schaken de stelling waarin een speler niet schaak staat, maar geen enkele geldige zet meer heeft? Het is remise.</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Pat</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr"/>
+      <c r="F48" s="9" t="inlineStr"/>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>?stalemate chess</t>
+        </is>
+      </c>
+      <c r="H48" s="6" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Schaken: rekensysteem voor de speelsterkte</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet het ratingsysteem voor de speelsterkte van schakers, genoemd naar een Hongaars-Amerikaanse natuurkundige?</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Elo</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr"/>
+      <c r="F49" s="9" t="inlineStr"/>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>Arpad Elo</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>Enige Nederlandse wereldkampioen schaken (1935)</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>Deze wiskundeleraar versloeg in 1935 Aljechin en werd de enige Nederlandse wereldkampioen schaken. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Max Euwe</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr"/>
+      <c r="F50" s="9" t="inlineStr"/>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>Max Euwe</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Noorse schaker, vijfvoudig wereldkampioen</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Deze Noorse schaker werd vijf keer wereldkampioen en haalde de hoogste rating ooit, 2882. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Magnus Carlsen</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr"/>
+      <c r="F51" s="9" t="inlineStr"/>
+      <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>Magnus Carlsen</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>Schaakcomputer die Kasparov in 1997 versloeg</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heette de schaakcomputer van IBM die in 1997 wereldkampioen Garri Kasparov in een match versloeg?</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>Deep Blue</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr"/>
+      <c r="F52" s="9" t="inlineStr"/>
+      <c r="G52" s="8" t="inlineStr">
+        <is>
+          <t>Deep Blue (schaakcomputer)</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Golf: één slag onder par</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het golf een hole die je in één slag minder dan par speelt, genoemd naar een vogeltje?</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Birdie</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Eagle = twee onder par, albatros = drie onder</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr"/>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>?birdie golf</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>Golf: twee slagen onder par</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het golf een hole die je in twee slagen minder dan par speelt, genoemd naar een roofvogel?</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Eagle</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr"/>
+      <c r="F54" s="9" t="inlineStr"/>
+      <c r="G54" s="8" t="inlineStr">
+        <is>
+          <t>?eagle golf score</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Golf: één slag boven par</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het golf een hole die je in één slag meer dan par speelt?</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Bogey</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr"/>
+      <c r="F55" s="9" t="inlineStr"/>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>?bogey golf</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Golf: tweejaarlijkse landenwedstrijd VS tegen Europa</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de tweejaarlijkse golfwedstrijd tussen teams uit de Verenigde Staten en Europa, genoemd naar een Engelse zaadhandelaar?</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Ryder Cup</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr"/>
+      <c r="F56" s="9" t="inlineStr"/>
+      <c r="G56" s="8" t="inlineStr">
+        <is>
+          <t>Ryder Cup</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Schaatsen: schaats met scharnier, revolutie eind jaren '90</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Deze schaats, met een scharnier aan de voorkant zodat het ijzer langer contact houdt met het ijs, veroorzaakte eind jaren negentig een revolutie in het langebaanschaatsen. Hoe heet hij?</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>Klapschaats</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr"/>
+      <c r="F57" s="9" t="inlineStr"/>
+      <c r="G57" s="8" t="inlineStr">
+        <is>
+          <t>Klapschaats</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>Schaatscoach van Wennemars en Kjeld Nuis, Gold Rush</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse schaatscoach leidt al decennia topploegen, met onder anderen Erben Wennemars en Kjeld Nuis. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Jac Orie</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr"/>
+      <c r="F58" s="9" t="inlineStr"/>
+      <c r="G58" s="8" t="inlineStr">
+        <is>
+          <t>Jac Orie</t>
+        </is>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Schaatscoach van Yvonne van Gennep en Marianne Timmer</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse schaatscoach begeleidde Yvonne van Gennep naar drie olympische titels in Calgary 1988 en later Marianne Timmer. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Egbert van 't Oever</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr"/>
+      <c r="F59" s="9" t="inlineStr"/>
+      <c r="G59" s="8" t="inlineStr">
+        <is>
+          <t>Egbert van 't Oever</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Coach van Sven Kramer, foute wissel Vancouver 2010</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse schaatscoach stuurde Sven Kramer in Vancouver 2010 op de 10.000 meter de verkeerde baan in, waardoor zijn pupil werd gediskwalificeerd. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Gerard Kemkers</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr"/>
+      <c r="F60" s="9" t="inlineStr"/>
+      <c r="G60" s="8" t="inlineStr">
+        <is>
+          <t>Gerard Kemkers</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Allrounder uit Lekkerkerk, drievoudig wereldkampioen</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Deze langebaanschaatser uit Lekkerkerk, zoon van een boer, werd drie keer achter elkaar wereldkampioen allround. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Patrick Roest</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>Niet: Marcel Bosker, Beau Snellink</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="inlineStr"/>
+      <c r="G61" s="8" t="inlineStr">
+        <is>
+          <t>Patrick Roest</t>
+        </is>
+      </c>
+      <c r="H61" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>Amerikaanse schaatswonder uit Wisconsin</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>Deze jonge Amerikaanse schaatser uit Wisconsin won in 2023 en 2024 op de WK afstanden goud op de 500, 1000 en 1500 meter en kreeg de Oscar Mathisen-trofee. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D62" s="8" t="inlineStr">
+        <is>
+          <t>Jordan Stolz</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr"/>
+      <c r="F62" s="9" t="inlineStr"/>
+      <c r="G62" s="8" t="inlineStr">
+        <is>
+          <t>Jordan Stolz</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Noorse schaatser, 5000 meter onder zes minuten</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Deze Noorse langebaanschaatser reed als eerste de 5000 meter onder de zes minuten en werd olympisch kampioen in Milaan. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Sander Eitrem</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr"/>
+      <c r="F63" s="9" t="inlineStr"/>
+      <c r="G63" s="8" t="inlineStr">
+        <is>
+          <t>Sander Eitrem</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>Japanse schaatsster, WR 1500 m, Nederlandse coach</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>Deze Japanse langebaanschaatster heeft het wereldrecord op de 1500 meter, reed bij de Nederlandse ploeg Team Gold en had een Nederlandse coach. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Miho Takagi</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr"/>
+      <c r="F64" s="9" t="inlineStr"/>
+      <c r="G64" s="8" t="inlineStr">
+        <is>
+          <t>Miho Takagi</t>
+        </is>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Zweedse schaatser, olympisch goud 5 en 10 km in 2022</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Deze Zweedse schaatser won in 2022 olympisch goud op de 5 en 10 kilometer en maakte daarna zijn hele trainingsschema openbaar. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Nils van der Poel</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr"/>
+      <c r="F65" s="9" t="inlineStr"/>
+      <c r="G65" s="8" t="inlineStr">
+        <is>
+          <t>Nils van der Poel</t>
+        </is>
+      </c>
+      <c r="H65" s="6" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>Drievoudig olympisch kampioen 2022 (3, 5 km, massastart)</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>Deze Noord-Hollandse schaatsster won op de Spelen van 2022 goud op de 3000 meter, de 5000 meter en de massastart. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Irene Schouten</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr"/>
+      <c r="F66" s="9" t="inlineStr"/>
+      <c r="G66" s="8" t="inlineStr">
+        <is>
+          <t>Irene Schouten</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Meest succesvolle Nederlandse olympiër, vijf Spelen goud</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Deze schaatsster won op vijf achtereenvolgende Olympische Spelen goud en is met dertien medailles de meest succesvolle Nederlandse olympiër. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>Ireen Wüst</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr"/>
+      <c r="F67" s="9" t="inlineStr"/>
+      <c r="G67" s="8" t="inlineStr">
+        <is>
+          <t>Ireen Wüst</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Drie olympische titels Sapporo 1972</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse schaatser won in 1972 in Sapporo drie olympische titels en werd ook drie keer wereldkampioen allround. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Ard Schenk</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr"/>
+      <c r="F68" s="9" t="inlineStr"/>
+      <c r="G68" s="8" t="inlineStr">
+        <is>
+          <t>Ard Schenk</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Shorttrackster, olympisch kampioen 1000 m 2018</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse shorttrackster werd in 2018 olympisch kampioen op de 1000 meter en later meervoudig wereldkampioen. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Suzanne Schulting</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr"/>
+      <c r="F69" s="9" t="inlineStr"/>
+      <c r="G69" s="8" t="inlineStr">
+        <is>
+          <t>Suzanne Schulting</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>Fries balspel, PC in Franeker</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>In dit Friese balspel slaan partuurs van drie spelers een bal met de hand, met 'kaatsen' en 'boppeslaan'. Het belangrijkste toernooi is de PC. In welke stad wordt de PC gespeeld?</t>
+        </is>
+      </c>
+      <c r="D70" s="8" t="inlineStr">
+        <is>
+          <t>Franeker</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr"/>
+      <c r="F70" s="9" t="inlineStr"/>
+      <c r="G70" s="8" t="inlineStr">
+        <is>
+          <t>!Franeker</t>
+        </is>
+      </c>
+      <c r="H70" s="6" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>Friese sport: met een polsstok over een sloot</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>In deze Friese sport klimmen springers in een lange stok terwijl die over een sloot kantelt, en landen ze aan de overkant in het zand. Hoe heet de sport?</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Fierljeppen</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr"/>
+      <c r="F71" s="9" t="inlineStr"/>
+      <c r="G71" s="8" t="inlineStr">
+        <is>
+          <t>Fierljeppen</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>Twentse sport: bal met lood zo ver mogelijk gooien over wegen</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>In deze Twentse en Achterhoekse sport gooien teams een met lood gevulde houten bal over landwegen; wie het minst aantal worpen nodig heeft, wint. Hoe heet hij?</t>
+        </is>
+      </c>
+      <c r="D72" s="8" t="inlineStr">
+        <is>
+          <t>Klootschieten</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr"/>
+      <c r="F72" s="9" t="inlineStr"/>
+      <c r="G72" s="8" t="inlineStr">
+        <is>
+          <t>Klootschieten</t>
+        </is>
+      </c>
+      <c r="H72" s="6" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>Nederlandse balsport uit 1902, gemengde teams</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Deze balsport werd in 1902 in Amsterdam bedacht door onderwijzer Nico Broekhuysen en wordt gespeeld in gemengde teams van mannen en vrouwen. Hoe heet hij?</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>Korfbal</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr"/>
+      <c r="F73" s="9" t="inlineStr"/>
+      <c r="G73" s="8" t="inlineStr">
+        <is>
+          <t>Korfbal</t>
+        </is>
+      </c>
+      <c r="H73" s="6" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>Wintersport: met het hoofd vooruit op een slee</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>Bij deze olympische wintersport ligt de sporter op de buik met het hoofd vooruit op een kleine slee en raast door een ijsbaan. Hoe heet hij?</t>
+        </is>
+      </c>
+      <c r="D74" s="8" t="inlineStr">
+        <is>
+          <t>Skeleton</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>Rodelen = op de rug, voeten vooruit</t>
+        </is>
+      </c>
+      <c r="F74" s="9" t="inlineStr"/>
+      <c r="G74" s="8" t="inlineStr">
+        <is>
+          <t>?skeleton sled</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Wintersport: langlaufen en schieten</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Deze olympische wintersport combineert langlaufen met geweerschieten. Hoe heet hij?</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>Biatlon</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr"/>
+      <c r="F75" s="9" t="inlineStr"/>
+      <c r="G75" s="8" t="inlineStr">
+        <is>
+          <t>Biatlon</t>
+        </is>
+      </c>
+      <c r="H75" s="6" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>Wintersport met stenen en vegen</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>Bij deze olympische wintersport schuiven teams granieten stenen over het ijs naar een doel, terwijl teamgenoten het ijs voor de steen vegen. Hoe heet hij?</t>
+        </is>
+      </c>
+      <c r="D76" s="8" t="inlineStr">
+        <is>
+          <t>Curling</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr"/>
+      <c r="F76" s="9" t="inlineStr"/>
+      <c r="G76" s="8" t="inlineStr">
+        <is>
+          <t>Curling</t>
+        </is>
+      </c>
+      <c r="H76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Biljart met drie ballen zonder zakken</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de vorm van biljart met drie ballen en een tafel zonder zakken, waarbij je met je speelbal beide andere ballen moet raken?</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>Carambole</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr"/>
+      <c r="F77" s="9" t="inlineStr"/>
+      <c r="G77" s="8" t="inlineStr">
+        <is>
+          <t>?carambole billiards</t>
+        </is>
+      </c>
+      <c r="H77" s="6" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B78" s="7" t="inlineStr">
+        <is>
+          <t>Schermen: wapen waarbij het hele lichaam trefvlak is</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>Bij het schermen zijn er drie wapens: floret, sabel en nog een, waarbij het hele lichaam trefvlak is. Welk wapen?</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>Degen</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr"/>
+      <c r="F78" s="9" t="inlineStr"/>
+      <c r="G78" s="8" t="inlineStr">
+        <is>
+          <t>?épée fencing</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Boksen: opwaartse stoot naar de kin</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet in het boksen een opwaartse stoot van onderen naar de kin?</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="inlineStr">
+        <is>
+          <t>Uppercut</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr"/>
+      <c r="F79" s="9" t="inlineStr"/>
+      <c r="G79" s="8" t="inlineStr">
+        <is>
+          <t>Uppercut</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B80" s="7" t="inlineStr">
+        <is>
+          <t>Bokspartij Ali vs Frazier, Filipijnen 1975</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>Hoe noemden de media de beroemde bokspartij tussen Muhammad Ali en Joe Frazier in 1975 in de Filipijnen, die veertien ronden duurde?</t>
+        </is>
+      </c>
+      <c r="D80" s="8" t="inlineStr">
+        <is>
+          <t>Thrilla in Manila</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr"/>
+      <c r="F80" s="9" t="inlineStr"/>
+      <c r="G80" s="8" t="inlineStr">
+        <is>
+          <t>Thrilla in Manila</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Bokspartij Ali vs Foreman, Kinshasa 1974</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Hoe noemden de media de bokspartij tussen Muhammad Ali en George Foreman in 1974 in Kinshasa, Zaïre?</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="inlineStr">
+        <is>
+          <t>Rumble in the Jungle</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr"/>
+      <c r="F81" s="9" t="inlineStr"/>
+      <c r="G81" s="8" t="inlineStr">
+        <is>
+          <t>Rumble in the Jungle</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>Amerikaanse YouTuber-bokser, verloofd met Jutta Leerdam</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>Deze Amerikaanse YouTuber werd bokser, vocht tegen Mike Tyson en is verloofd met schaatsster Jutta Leerdam. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>Jake Paul</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr"/>
+      <c r="F82" s="9" t="inlineStr"/>
+      <c r="G82" s="8" t="inlineStr">
+        <is>
+          <t>Jake Paul</t>
+        </is>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Nederlandse kickbokser, Glory-kampioen zwaargewicht</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse kickbokser was jarenlang wereldkampioen zwaargewicht van de organisatie Glory. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="inlineStr">
+        <is>
+          <t>Rico Verhoeven</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr"/>
+      <c r="F83" s="9" t="inlineStr"/>
+      <c r="G83" s="8" t="inlineStr">
+        <is>
+          <t>Rico Verhoeven</t>
+        </is>
+      </c>
+      <c r="H83" s="6" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>Beste Nederlandse tennisser, toernooiwinst Rosmalen 2023</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse tennisser stond 21e op de wereldranglijst en won in 2023 het grastoernooi van Rosmalen. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D84" s="8" t="inlineStr">
+        <is>
+          <t>Tallon Griekspoor</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>Niet: Botic van de Zandschulp</t>
+        </is>
+      </c>
+      <c r="F84" s="9" t="inlineStr"/>
+      <c r="G84" s="8" t="inlineStr">
+        <is>
+          <t>Tallon Griekspoor</t>
+        </is>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Tennisser die Nadal zijn laatste partij liet verliezen (2024)</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse tennisser versloeg in 2024 op de US Open Carlos Alcaraz, en won later dat jaar in de Davis Cup de allerlaatste partij van Rafael Nadal. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>Botic van de Zandschulp</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr"/>
+      <c r="F85" s="9" t="inlineStr"/>
+      <c r="G85" s="8" t="inlineStr">
+        <is>
+          <t>Botic van de Zandschulp</t>
+        </is>
+      </c>
+      <c r="H85" s="6" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>Nederlandse Wimbledon-winnaar 1996</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse tennisser won in 1996 als enige Nederlander het herenenkel op Wimbledon. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>Richard Krajicek</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="inlineStr"/>
+      <c r="F86" s="9" t="inlineStr"/>
+      <c r="G86" s="8" t="inlineStr">
+        <is>
+          <t>Richard Krajicek</t>
+        </is>
+      </c>
+      <c r="H86" s="6" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Rolstoeltennisster, 470 partijen ongeslagen</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse rolstoeltennisster bleef tien jaar lang ongeslagen en won 470 partijen op rij. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>Esther Vergeer</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr"/>
+      <c r="F87" s="9" t="inlineStr"/>
+      <c r="G87" s="8" t="inlineStr">
+        <is>
+          <t>Esther Vergeer</t>
+        </is>
+      </c>
+      <c r="H87" s="6" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>Rolstoeltennisster, Golden Slam 2021</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse rolstoeltennisster won in 2021 alle vier de grandslams én olympisch goud, de Golden Slam. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D88" s="8" t="inlineStr">
+        <is>
+          <t>Diede de Groot</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="inlineStr"/>
+      <c r="F88" s="9" t="inlineStr"/>
+      <c r="G88" s="8" t="inlineStr">
+        <is>
+          <t>Diede de Groot</t>
+        </is>
+      </c>
+      <c r="H88" s="6" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>Agassi's rivaal, 14 grandslams</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>Deze Amerikaanse tennisser was de grote rivaal van Andre Agassi en won veertien grandslamtitels, de laatste op de US Open van 2002. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>Pete Sampras</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="inlineStr"/>
+      <c r="F89" s="9" t="inlineStr"/>
+      <c r="G89" s="8" t="inlineStr">
+        <is>
+          <t>Pete Sampras</t>
+        </is>
+      </c>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>Poolse tennisster, meervoudig winnares Roland Garros</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>Deze Poolse tennisster won meerdere keren Roland Garros en stond lang nummer één van de wereld. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D90" s="8" t="inlineStr">
+        <is>
+          <t>Iga Świątek</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr"/>
+      <c r="F90" s="9" t="inlineStr"/>
+      <c r="G90" s="8" t="inlineStr">
+        <is>
+          <t>Iga Świątek</t>
+        </is>
+      </c>
+      <c r="H90" s="6" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>Nederlandse marathonloper, won New York 2024</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse marathonloper, geboren in Somalië, won zilver op de Spelen van Tokio en won in 2024 de marathon van New York. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>Abdi Nageeye</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr"/>
+      <c r="F91" s="9" t="inlineStr"/>
+      <c r="G91" s="8" t="inlineStr">
+        <is>
+          <t>Abdi Nageeye</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>Sprinter uit Zoetermeer, olympisch goud gemengde 4x400 m</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse sprinter uit Zoetermeer met Oegandese wortels liep in 2024 mee in de gemengde estafetteploeg op de 4x400 meter die olympisch goud won. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D92" s="8" t="inlineStr">
+        <is>
+          <t>Eugene Omalla</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr"/>
+      <c r="F92" s="9" t="inlineStr"/>
+      <c r="G92" s="8" t="inlineStr">
+        <is>
+          <t>Eugene Omalla</t>
+        </is>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>Zweeds-Amerikaanse polsstokhoogspringer, wereldrecords</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>Deze Zweeds-Amerikaanse atleet verbeterde het wereldrecord polsstokhoogspringen keer op keer, tot boven de 6,30 meter. Wat is zijn bijnaam, waaronder iedereen hem kent?</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="inlineStr">
+        <is>
+          <t>Mondo</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>Armand Duplantis</t>
+        </is>
+      </c>
+      <c r="F93" s="9" t="inlineStr"/>
+      <c r="G93" s="8" t="inlineStr">
+        <is>
+          <t>Armand Duplantis</t>
+        </is>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>Hoogspringtechniek met de rug over de lat</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr">
+        <is>
+          <t>Deze Amerikaanse hoogspringer won in 1968 olympisch goud met een nieuwe techniek waarbij je met je rug over de lat gaat, die nu naar hem is genoemd. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D94" s="8" t="inlineStr">
+        <is>
+          <t>Fosbury</t>
+        </is>
+      </c>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>Dick Fosbury, de 'Fosbury flop'</t>
+        </is>
+      </c>
+      <c r="F94" s="9" t="inlineStr"/>
+      <c r="G94" s="8" t="inlineStr">
+        <is>
+          <t>Dick Fosbury</t>
+        </is>
+      </c>
+      <c r="H94" s="6" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>Olympisch goud marathon Parijs 2024, ook 5 en 10 km</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse atlete won in Parijs 2024 brons op de 5 en de 10 kilometer en daarna goud op de marathon. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="inlineStr">
+        <is>
+          <t>Sifan Hassan</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="inlineStr"/>
+      <c r="F95" s="9" t="inlineStr"/>
+      <c r="G95" s="8" t="inlineStr">
+        <is>
+          <t>Sifan Hassan</t>
+        </is>
+      </c>
+      <c r="H95" s="6" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B96" s="7" t="inlineStr">
+        <is>
+          <t>Brabantse baanwielrenner, keirin en sprint</t>
+        </is>
+      </c>
+      <c r="C96" s="7" t="inlineStr">
+        <is>
+          <t>Deze Brabantse baansprinter werd vele malen wereldkampioen en won meerdere keren olympisch goud, onder meer op de keirin. Wie is hij?</t>
+        </is>
+      </c>
+      <c r="D96" s="8" t="inlineStr">
+        <is>
+          <t>Harrie Lavreysen</t>
+        </is>
+      </c>
+      <c r="E96" s="7" t="inlineStr"/>
+      <c r="F96" s="9" t="inlineStr"/>
+      <c r="G96" s="8" t="inlineStr">
+        <is>
+          <t>Harrie Lavreysen</t>
+        </is>
+      </c>
+      <c r="H96" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>Wielrenster: mountainbike-WK en Tour de France</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>Deze Nederlandse wielrenster werd wereldkampioen mountainbike en reed ook de Tour de France Femmes. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="inlineStr">
+        <is>
+          <t>Puck Pieterse</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="inlineStr"/>
+      <c r="F97" s="9" t="inlineStr"/>
+      <c r="G97" s="8" t="inlineStr">
+        <is>
+          <t>Puck Pieterse</t>
+        </is>
+      </c>
+      <c r="H97" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B98" s="7" t="inlineStr">
+        <is>
+          <t>Belgische wielrenster, WK op weg en baan</t>
+        </is>
+      </c>
+      <c r="C98" s="7" t="inlineStr">
+        <is>
+          <t>Deze Belgische wielrenster werd wereldkampioen op de weg en op de baan en won de Ronde van Vlaanderen. Wie is zij?</t>
+        </is>
+      </c>
+      <c r="D98" s="8" t="inlineStr">
+        <is>
+          <t>Lotte Kopecky</t>
+        </is>
+      </c>
+      <c r="E98" s="7" t="inlineStr"/>
+      <c r="F98" s="9" t="inlineStr"/>
+      <c r="G98" s="8" t="inlineStr">
+        <is>
+          <t>Lotte Kopecky</t>
+        </is>
+      </c>
+      <c r="H98" s="6" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>Grote drafwedstrijd op de renbaan van Vincennes</t>
+        </is>
+      </c>
+      <c r="C99" s="7" t="inlineStr">
+        <is>
+          <t>Hoe heet de belangrijkste drafwedstrijd ter wereld, die elk jaar in januari op de renbaan van Vincennes bij Parijs wordt verreden?</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="inlineStr">
+        <is>
+          <t>Prix d'Amérique</t>
+        </is>
+      </c>
+      <c r="E99" s="7" t="inlineStr"/>
+      <c r="F99" s="9" t="inlineStr"/>
+      <c r="G99" s="8" t="inlineStr">
+        <is>
+          <t>Prix d'Amérique</t>
+        </is>
+      </c>
+      <c r="H99" s="6" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>